<commit_message>
Chap 5, EX 3
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{8CE6D65F-09EE-4825-B192-E5363BB813BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D657E3-4821-4394-9C10-39EF8718EB63}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{8CE6D65F-09EE-4825-B192-E5363BB813BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{284EC2BB-6BE7-4D0E-A6C9-B002A69A682E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="151">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -485,10 +485,14 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Actual done: 2026-01-31</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-01</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -653,6 +657,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1045,10 +1053,10 @@
         <v>46055</v>
       </c>
       <c r="I5" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J5" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="K5" s="6"/>
     </row>
@@ -1078,10 +1086,10 @@
         <v>46056</v>
       </c>
       <c r="I6" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="K6" s="6"/>
     </row>
@@ -1104,14 +1112,18 @@
         <v>60</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="7" t="str">
+        <v>147</v>
+      </c>
+      <c r="H7" s="7">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
+        <v>46057</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.15">
@@ -3445,7 +3457,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3463,7 +3475,7 @@
       </c>
       <c r="B8" s="12">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3488,7 +3500,7 @@
       </c>
       <c r="B12" s="12">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
@@ -3497,11 +3509,12 @@
       </c>
       <c r="B13" s="12">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, EX 5(c)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{8CE6D65F-09EE-4825-B192-E5363BB813BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{284EC2BB-6BE7-4D0E-A6C9-B002A69A682E}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{8CE6D65F-09EE-4825-B192-E5363BB813BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F662BBD0-1442-4D5F-9EC2-05012B0DE679}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6015" yWindow="1830" windowWidth="22095" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="155">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -489,11 +489,24 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Actual done: 2026-02-01</t>
     <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-02</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual not started: 2026-02-02</t>
+  </si>
+  <si>
+    <t>Actual not started: 2026-02-12</t>
+  </si>
+  <si>
+    <t>Actual not started: 2026-02-22</t>
   </si>
 </sst>
 </file>
@@ -1053,7 +1066,7 @@
         <v>46055</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>148</v>
@@ -1086,7 +1099,7 @@
         <v>46056</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>148</v>
@@ -1119,10 +1132,10 @@
         <v>46057</v>
       </c>
       <c r="I7" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="J7" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>150</v>
       </c>
       <c r="K7" s="6"/>
     </row>
@@ -1145,14 +1158,16 @@
         <v>60</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="7" t="str">
+        <v>147</v>
+      </c>
+      <c r="H8" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46058</v>
       </c>
       <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>151</v>
+      </c>
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.15">
@@ -3457,7 +3472,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3475,7 +3490,7 @@
       </c>
       <c r="B8" s="12">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3500,7 +3515,7 @@
       </c>
       <c r="B12" s="12">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
@@ -3509,7 +3524,7 @@
       </c>
       <c r="B13" s="12">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chap 5, EX 6(C), 10
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9224FD5-EDFF-4B56-9155-F708E0ADFF3E}"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7785"/>
+    <workbookView xWindow="6015" yWindow="1830" windowWidth="22095" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -15,12 +21,25 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Plan'!$A$4:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercise Map'!$A$3:$F$43</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="156">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -106,10 +125,7 @@
     <t>Exercises: Ex6(a–c) (L1)</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>(a): 2026-02-04</t>
+    <t>(a)(b): 2026-02-04</t>
   </si>
   <si>
     <t>Exercises: Ex10 (L1) + 10-min recap note</t>
@@ -485,20 +501,24 @@
   </si>
   <si>
     <t>C1 Marked Yes</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-05</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>(a)(b): 2026-02-04, © 2026-02-05</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -532,151 +552,22 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <sz val="9"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -695,194 +586,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -905,338 +610,53 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1250,7 +670,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1259,6 +679,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1543,14 +966,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1564,12 +987,22 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" spans="1:1">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1583,46 +1016,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="27" spans="1:11">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="11">
         <f t="shared" ref="B5:B36" si="0">IF($B$2="","",$B$2+A5-1)</f>
         <v>46053</v>
       </c>
@@ -1639,7 +1072,7 @@
       <c r="G5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="12">
         <f t="shared" ref="H5:H36" si="1">IF(G5="Done",B5+2,"")</f>
         <v>46055</v>
       </c>
@@ -1651,11 +1084,11 @@
       </c>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A6" s="10">
         <v>2</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>46054</v>
       </c>
@@ -1672,7 +1105,7 @@
       <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="12">
         <f t="shared" si="1"/>
         <v>46056</v>
       </c>
@@ -1684,11 +1117,11 @@
       </c>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A7" s="10">
         <v>3</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="11">
         <f t="shared" si="0"/>
         <v>46055</v>
       </c>
@@ -1705,7 +1138,7 @@
       <c r="G7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <f t="shared" si="1"/>
         <v>46057</v>
       </c>
@@ -1717,11 +1150,11 @@
       </c>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A8" s="10">
         <v>4</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>46056</v>
       </c>
@@ -1738,7 +1171,7 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="12">
         <f t="shared" si="1"/>
         <v>46058</v>
       </c>
@@ -1748,11 +1181,11 @@
       </c>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A9" s="10">
         <v>5</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="11">
         <f t="shared" si="0"/>
         <v>46057</v>
       </c>
@@ -1769,7 +1202,7 @@
       <c r="G9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <f t="shared" si="1"/>
         <v>46059</v>
       </c>
@@ -1779,11 +1212,11 @@
       </c>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="11">
+    <row r="10" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A10" s="10">
         <v>6</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>46058</v>
       </c>
@@ -1798,23 +1231,23 @@
         <v>90</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H10" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46060</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="8" t="s">
-        <v>29</v>
+      <c r="J10" s="16" t="s">
+        <v>155</v>
       </c>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A11" s="10">
         <v>7</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="11">
         <f t="shared" si="0"/>
         <v>46059</v>
       </c>
@@ -1823,46 +1256,48 @@
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F11" s="8">
         <v>60</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H11" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46061</v>
       </c>
       <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="J11" s="16" t="s">
+        <v>154</v>
+      </c>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A12" s="10">
         <v>8</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>46060</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="F12" s="8">
         <v>75</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H12" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1870,30 +1305,30 @@
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A13" s="10">
         <v>9</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="11">
         <f t="shared" si="0"/>
         <v>46061</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="F13" s="8">
         <v>75</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H13" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1901,28 +1336,28 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A14" s="10">
         <v>10</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>46062</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F14" s="8">
         <v>60</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H14" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1930,28 +1365,28 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A15" s="10">
         <v>11</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <f t="shared" si="0"/>
         <v>46063</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F15" s="8">
         <v>90</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H15" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H15" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1959,28 +1394,28 @@
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A16" s="10">
         <v>12</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>46064</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F16" s="8">
         <v>90</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H16" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H16" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1988,28 +1423,28 @@
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A17" s="10">
         <v>13</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <f t="shared" si="0"/>
         <v>46065</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F17" s="8">
         <v>90</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H17" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H17" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2017,28 +1452,28 @@
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" ht="27" spans="1:11">
-      <c r="A18" s="11">
+    <row r="18" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A18" s="10">
         <v>14</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <f t="shared" si="0"/>
         <v>46066</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F18" s="8">
         <v>45</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H18" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H18" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2046,30 +1481,30 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A19" s="10">
         <v>15</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="11">
         <f t="shared" si="0"/>
         <v>46067</v>
       </c>
       <c r="C19" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="E19" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="F19" s="8">
         <v>75</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H19" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2077,28 +1512,28 @@
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A20" s="10">
         <v>16</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>46068</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F20" s="8">
         <v>60</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H20" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H20" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2106,30 +1541,30 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A21" s="10">
         <v>17</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="11">
         <f t="shared" si="0"/>
         <v>46069</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>48</v>
       </c>
       <c r="F21" s="8">
         <v>75</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H21" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H21" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2137,28 +1572,28 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A22" s="10">
         <v>18</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>46070</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F22" s="8">
         <v>90</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H22" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H22" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2166,28 +1601,28 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A23" s="10">
         <v>19</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="11">
         <f t="shared" si="0"/>
         <v>46071</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F23" s="8">
         <v>90</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H23" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H23" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2195,28 +1630,28 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A24" s="10">
         <v>20</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="11">
         <f t="shared" si="0"/>
         <v>46072</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F24" s="8">
         <v>90</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H24" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H24" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2224,28 +1659,28 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A25" s="10">
         <v>21</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="11">
         <f t="shared" si="0"/>
         <v>46073</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F25" s="8">
         <v>60</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H25" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H25" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2253,30 +1688,30 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A26" s="10">
         <v>22</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>46074</v>
       </c>
       <c r="C26" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>56</v>
       </c>
       <c r="F26" s="8">
         <v>75</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H26" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H26" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2284,28 +1719,28 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A27" s="10">
         <v>23</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="11">
         <f t="shared" si="0"/>
         <v>46075</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F27" s="8">
         <v>45</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H27" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H27" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2313,30 +1748,30 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A28" s="10">
         <v>24</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>46076</v>
       </c>
       <c r="C28" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="E28" s="8" t="s">
         <v>59</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>60</v>
       </c>
       <c r="F28" s="8">
         <v>75</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H28" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H28" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2344,28 +1779,28 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A29" s="10">
         <v>25</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="11">
         <f t="shared" si="0"/>
         <v>46077</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F29" s="8">
         <v>90</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H29" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H29" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2373,28 +1808,28 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A30" s="10">
         <v>26</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>46078</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F30" s="8">
         <v>90</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H30" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H30" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2402,28 +1837,28 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A31" s="10">
         <v>27</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="11">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F31" s="8">
         <v>75</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H31" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H31" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2431,28 +1866,28 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A32" s="10">
         <v>28</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>46080</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F32" s="8">
         <v>45</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H32" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H32" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2460,30 +1895,30 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A33" s="10">
         <v>29</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="11">
         <f t="shared" si="0"/>
         <v>46081</v>
       </c>
       <c r="C33" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>69</v>
       </c>
       <c r="F33" s="8">
         <v>75</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H33" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H33" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2491,28 +1926,28 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="11">
-        <v>30</v>
-      </c>
-      <c r="B34" s="12">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A34" s="10">
+        <v>30</v>
+      </c>
+      <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>46082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F34" s="8">
         <v>75</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H34" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H34" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2520,28 +1955,28 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A35" s="10">
         <v>31</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="11">
         <f t="shared" si="0"/>
         <v>46083</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F35" s="8">
         <v>60</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H35" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H35" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2549,28 +1984,28 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A36" s="10">
         <v>32</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="11">
         <f t="shared" si="0"/>
         <v>46084</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F36" s="8">
         <v>90</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H36" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H36" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2578,30 +2013,30 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A37" s="10">
         <v>33</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="11">
         <f t="shared" ref="B37:B56" si="2">IF($B$2="","",$B$2+A37-1)</f>
         <v>46085</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D37" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>75</v>
       </c>
       <c r="F37" s="8">
         <v>90</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H37" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H37" s="12" t="str">
         <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
         <v/>
       </c>
@@ -2609,30 +2044,30 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A38" s="10">
         <v>34</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="11">
         <f t="shared" si="2"/>
         <v>46086</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D38" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>77</v>
       </c>
       <c r="F38" s="8">
         <v>90</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H38" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H38" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2640,28 +2075,28 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A39" s="10">
         <v>35</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="11">
         <f t="shared" si="2"/>
         <v>46087</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F39" s="8">
         <v>60</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H39" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H39" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2669,28 +2104,28 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11">
-      <c r="A40" s="11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A40" s="10">
         <v>36</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="11">
         <f t="shared" si="2"/>
         <v>46088</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F40" s="8">
         <v>90</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H40" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H40" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2698,28 +2133,28 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A41" s="10">
         <v>37</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="11">
         <f t="shared" si="2"/>
         <v>46089</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H41" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H41" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2727,28 +2162,28 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11">
-      <c r="A42" s="11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A42" s="10">
         <v>38</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="11">
         <f t="shared" si="2"/>
         <v>46090</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H42" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H42" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2756,28 +2191,28 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11">
-      <c r="A43" s="11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A43" s="10">
         <v>39</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="11">
         <f t="shared" si="2"/>
         <v>46091</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H43" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H43" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2785,28 +2220,28 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11">
-      <c r="A44" s="11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A44" s="10">
         <v>40</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="11">
         <f t="shared" si="2"/>
         <v>46092</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H44" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H44" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2814,28 +2249,28 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A45" s="10">
         <v>41</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="11">
         <f t="shared" si="2"/>
         <v>46093</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H45" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H45" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2843,28 +2278,28 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A46" s="10">
         <v>42</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="11">
         <f t="shared" si="2"/>
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H46" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H46" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2872,28 +2307,28 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11">
-      <c r="A47" s="11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A47" s="10">
         <v>43</v>
       </c>
-      <c r="B47" s="12">
+      <c r="B47" s="11">
         <f t="shared" si="2"/>
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H47" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H47" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2901,28 +2336,28 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11">
-      <c r="A48" s="11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A48" s="10">
         <v>44</v>
       </c>
-      <c r="B48" s="12">
+      <c r="B48" s="11">
         <f t="shared" si="2"/>
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H48" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H48" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2930,28 +2365,28 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11">
-      <c r="A49" s="11">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A49" s="10">
         <v>45</v>
       </c>
-      <c r="B49" s="12">
+      <c r="B49" s="11">
         <f t="shared" si="2"/>
         <v>46097</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H49" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H49" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2959,28 +2394,28 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11">
-      <c r="A50" s="11">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A50" s="10">
         <v>46</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="11">
         <f t="shared" si="2"/>
         <v>46098</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H50" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H50" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2988,11 +2423,11 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11">
-      <c r="A51" s="11">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A51" s="10">
         <v>47</v>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="11">
         <f t="shared" si="2"/>
         <v>46099</v>
       </c>
@@ -3001,15 +2436,15 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H51" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H51" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3017,28 +2452,28 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11">
-      <c r="A52" s="11">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A52" s="10">
         <v>48</v>
       </c>
-      <c r="B52" s="12">
+      <c r="B52" s="11">
         <f t="shared" si="2"/>
         <v>46100</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H52" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H52" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3046,28 +2481,28 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11">
-      <c r="A53" s="11">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A53" s="10">
         <v>49</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="11">
         <f t="shared" si="2"/>
         <v>46101</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H53" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H53" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3075,28 +2510,28 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11">
-      <c r="A54" s="11">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A54" s="10">
         <v>50</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="11">
         <f t="shared" si="2"/>
         <v>46102</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H54" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H54" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3104,28 +2539,28 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="11">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A55" s="10">
         <v>51</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="11">
         <f t="shared" si="2"/>
         <v>46103</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H55" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H55" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3133,28 +2568,28 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" ht="27" spans="1:11">
-      <c r="A56" s="11">
+    <row r="56" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A56" s="10">
         <v>52</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="11">
         <f t="shared" si="2"/>
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H56" s="13" t="str">
+        <v>30</v>
+      </c>
+      <c r="H56" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3163,41 +2598,38 @@
       <c r="K56" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K56">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A4:K56" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A5:K56">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$G5="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>$G5="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$G5="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="I5:I56">
+    <dataValidation type="list" sqref="G5:G56" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"Not Started,In Progress,Done"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I5:I56" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"No,Yes"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="G5:G56">
-      <formula1>"Not Started,In Progress,Done"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -3207,49 +2639,54 @@
     <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A2" s="5" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="3" ht="27" spans="1:6">
+    <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>102</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>103</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A4" s="8">
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>104</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>105</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -3260,15 +2697,15 @@
       </c>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A5" s="8">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3279,15 +2716,15 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A6" s="8">
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -3298,15 +2735,15 @@
       </c>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A7" s="8">
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3317,15 +2754,15 @@
       </c>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" ht="27" spans="1:6">
+    <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A8" s="8">
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -3336,91 +2773,91 @@
       </c>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" ht="27" spans="1:6">
+    <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A9" s="8">
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A10" s="8">
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
         <v>2026-02-08</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A11" s="8">
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
         <v>2026-02-09</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A12" s="8">
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
         <v>2026-03-19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A13" s="8">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>114</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>115</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3431,509 +2868,509 @@
       </c>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A14" s="8">
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
         <v>2026-03-02</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" ht="27" spans="1:6">
+    <row r="15" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A15" s="8">
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
         <v>2026-02-24 – 2026-02-25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A16" s="8">
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
         <v>2026-02-10</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A17" s="8">
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
         <v>2026-02-16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A18" s="8">
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
         <v>2026-02-13</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" ht="27" spans="1:6">
+    <row r="19" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A19" s="8">
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A20" s="8">
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
         <v>2026-02-26</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A21" s="8">
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>124</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>125</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
         <v>2026-02-22</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A22" s="8">
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
         <v>2026-03-03</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" ht="27" spans="1:6">
+    <row r="23" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A23" s="8">
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
         <v>2026-02-17 – 2026-02-19</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A24" s="8">
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
         <v>2026-02-20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" ht="27" spans="1:6">
+    <row r="25" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A25" s="8">
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
         <v>2026-03-04 – 2026-03-07</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A26" s="8">
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
         <v>2026-02-23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A27" s="8">
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
         <v>2026-03-08</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" ht="27" spans="1:6">
+    <row r="28" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A28" s="8">
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
         <v>2026-03-16 – 2026-03-17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A29" s="8">
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
         <v>2026-03-11</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A30" s="8">
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
         <v>2026-02-27</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A31" s="8">
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
         <v>2026-03-10</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A32" s="8">
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
         <v>2026-03-12</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A33" s="8">
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
         <v>2026-02-11</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" ht="27" spans="1:6">
+    <row r="34" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A34" s="8">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A35" s="8">
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F35" s="8"/>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A36" s="8">
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F36" s="8"/>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A37" s="8">
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A38" s="8">
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
         <v>2026-03-09</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A39" s="8">
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
         <v>2026-02-12</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" s="8">
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3944,166 +3381,163 @@
       </c>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A41" s="8">
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
         <v>2026-02-07</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F41" s="8"/>
     </row>
-    <row r="42" ht="27" spans="1:6">
+    <row r="42" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A42" s="8">
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
         <v>2026-03-20 – 2026-03-21</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F42" s="8"/>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A43" s="8">
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
         <v>2026-03-22</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F43" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F43">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A3:F43" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:1">
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A3" s="2" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
@@ -4111,8 +3545,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, read 5.3
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9224FD5-EDFF-4B56-9155-F708E0ADFF3E}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35B6D921-4AD6-4932-811C-908664088637}"/>
   <bookViews>
     <workbookView xWindow="6015" yWindow="1830" windowWidth="22095" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="156">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>Exercises: Ex6(a–c) (L1)</t>
-  </si>
-  <si>
-    <t>(a)(b): 2026-02-04</t>
   </si>
   <si>
     <t>Exercises: Ex10 (L1) + 10-min recap note</t>
@@ -508,6 +505,10 @@
   </si>
   <si>
     <t>(a)(b): 2026-02-04, © 2026-02-05</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-06</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -516,7 +517,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -620,14 +621,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -638,16 +639,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -685,6 +686,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -988,19 +993,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
@@ -1238,8 +1243,8 @@
         <v>46060</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="16" t="s">
-        <v>155</v>
+      <c r="J10" s="13" t="s">
+        <v>154</v>
       </c>
       <c r="K10" s="8"/>
     </row>
@@ -1256,7 +1261,7 @@
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" s="8">
         <v>60</v>
@@ -1269,8 +1274,8 @@
         <v>46061</v>
       </c>
       <c r="I11" s="8"/>
-      <c r="J11" s="16" t="s">
-        <v>154</v>
+      <c r="J11" s="13" t="s">
+        <v>153</v>
       </c>
       <c r="K11" s="8"/>
     </row>
@@ -1283,26 +1288,28 @@
         <v>46060</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="8" t="s">
         <v>32</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>33</v>
       </c>
       <c r="F12" s="8">
         <v>75</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H12" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46062</v>
       </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="J12" s="13" t="s">
+        <v>155</v>
+      </c>
       <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.15">
@@ -1314,26 +1321,28 @@
         <v>46061</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D13" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>35</v>
       </c>
       <c r="F13" s="8">
         <v>75</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H13" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H13" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46063</v>
       </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="J13" s="13" t="s">
+        <v>155</v>
+      </c>
       <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.15">
@@ -1345,17 +1354,17 @@
         <v>46062</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F14" s="8">
         <v>60</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H14" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1374,17 +1383,17 @@
         <v>46063</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F15" s="8">
         <v>90</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H15" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1403,17 +1412,17 @@
         <v>46064</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F16" s="8">
         <v>90</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H16" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1432,17 +1441,17 @@
         <v>46065</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F17" s="8">
         <v>90</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H17" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1461,17 +1470,17 @@
         <v>46066</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F18" s="8">
         <v>45</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H18" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1490,19 +1499,19 @@
         <v>46067</v>
       </c>
       <c r="C19" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="E19" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="F19" s="8">
         <v>75</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H19" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1521,17 +1530,17 @@
         <v>46068</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F20" s="8">
         <v>60</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H20" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1550,19 +1559,19 @@
         <v>46069</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="F21" s="8">
         <v>75</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H21" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1581,17 +1590,17 @@
         <v>46070</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F22" s="8">
         <v>90</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H22" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1610,17 +1619,17 @@
         <v>46071</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F23" s="8">
         <v>90</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H23" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1639,17 +1648,17 @@
         <v>46072</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F24" s="8">
         <v>90</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H24" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1668,17 +1677,17 @@
         <v>46073</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F25" s="8">
         <v>60</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H25" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1697,19 +1706,19 @@
         <v>46074</v>
       </c>
       <c r="C26" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="8" t="s">
         <v>54</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>55</v>
       </c>
       <c r="F26" s="8">
         <v>75</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H26" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1728,17 +1737,17 @@
         <v>46075</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F27" s="8">
         <v>45</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H27" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1757,19 +1766,19 @@
         <v>46076</v>
       </c>
       <c r="C28" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="E28" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>59</v>
       </c>
       <c r="F28" s="8">
         <v>75</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H28" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1788,17 +1797,17 @@
         <v>46077</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F29" s="8">
         <v>90</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H29" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1817,17 +1826,17 @@
         <v>46078</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F30" s="8">
         <v>90</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H30" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1846,17 +1855,17 @@
         <v>46079</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F31" s="8">
         <v>75</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H31" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1875,17 +1884,17 @@
         <v>46080</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F32" s="8">
         <v>45</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H32" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1904,19 +1913,19 @@
         <v>46081</v>
       </c>
       <c r="C33" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>68</v>
       </c>
       <c r="F33" s="8">
         <v>75</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H33" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1935,17 +1944,17 @@
         <v>46082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F34" s="8">
         <v>75</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H34" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1964,17 +1973,17 @@
         <v>46083</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F35" s="8">
         <v>60</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H35" s="12" t="str">
         <f t="shared" si="1"/>
@@ -1993,17 +2002,17 @@
         <v>46084</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F36" s="8">
         <v>90</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H36" s="12" t="str">
         <f t="shared" si="1"/>
@@ -2022,19 +2031,19 @@
         <v>46085</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D37" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>74</v>
       </c>
       <c r="F37" s="8">
         <v>90</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H37" s="12" t="str">
         <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
@@ -2053,19 +2062,19 @@
         <v>46086</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D38" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>76</v>
       </c>
       <c r="F38" s="8">
         <v>90</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H38" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2084,17 +2093,17 @@
         <v>46087</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F39" s="8">
         <v>60</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H39" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2113,17 +2122,17 @@
         <v>46088</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F40" s="8">
         <v>90</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H40" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2142,17 +2151,17 @@
         <v>46089</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H41" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2171,17 +2180,17 @@
         <v>46090</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H42" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2200,17 +2209,17 @@
         <v>46091</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H43" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2229,17 +2238,17 @@
         <v>46092</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H44" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2258,17 +2267,17 @@
         <v>46093</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H45" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2287,17 +2296,17 @@
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H46" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2316,17 +2325,17 @@
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H47" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2345,17 +2354,17 @@
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H48" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2374,17 +2383,17 @@
         <v>46097</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H49" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2403,17 +2412,17 @@
         <v>46098</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H50" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2436,13 +2445,13 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H51" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2461,17 +2470,17 @@
         <v>46100</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H52" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2490,17 +2499,17 @@
         <v>46101</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H53" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2519,17 +2528,17 @@
         <v>46102</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H54" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2548,17 +2557,17 @@
         <v>46103</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H55" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2577,17 +2586,17 @@
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H56" s="12" t="str">
         <f t="shared" si="3"/>
@@ -2640,18 +2649,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="A1" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
@@ -2660,19 +2669,19 @@
     </row>
     <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
@@ -2683,10 +2692,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -2702,10 +2711,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2721,10 +2730,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -2740,10 +2749,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2759,10 +2768,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -2778,17 +2787,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -2797,17 +2806,17 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
         <v>2026-02-08</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -2816,17 +2825,17 @@
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
         <v>2026-02-09</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="8"/>
     </row>
@@ -2835,17 +2844,17 @@
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
         <v>2026-03-19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F12" s="8"/>
     </row>
@@ -2854,10 +2863,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>113</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -2873,17 +2882,17 @@
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
         <v>2026-03-02</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F14" s="8"/>
     </row>
@@ -2892,17 +2901,17 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
         <v>2026-02-24 – 2026-02-25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -2911,17 +2920,17 @@
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
         <v>2026-02-10</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="8"/>
     </row>
@@ -2930,17 +2939,17 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
         <v>2026-02-16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F17" s="8"/>
     </row>
@@ -2949,17 +2958,17 @@
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
         <v>2026-02-13</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F18" s="8"/>
     </row>
@@ -2968,17 +2977,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -2987,17 +2996,17 @@
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
         <v>2026-02-26</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -3006,17 +3015,17 @@
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
         <v>2026-02-22</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F21" s="8"/>
     </row>
@@ -3025,17 +3034,17 @@
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
         <v>2026-03-03</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F22" s="8"/>
     </row>
@@ -3044,17 +3053,17 @@
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
         <v>2026-02-17 – 2026-02-19</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F23" s="8"/>
     </row>
@@ -3063,17 +3072,17 @@
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
         <v>2026-02-20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F24" s="8"/>
     </row>
@@ -3082,17 +3091,17 @@
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
         <v>2026-03-04 – 2026-03-07</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F25" s="8"/>
     </row>
@@ -3101,17 +3110,17 @@
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
         <v>2026-02-23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F26" s="8"/>
     </row>
@@ -3120,17 +3129,17 @@
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
         <v>2026-03-08</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F27" s="8"/>
     </row>
@@ -3139,17 +3148,17 @@
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
         <v>2026-03-16 – 2026-03-17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F28" s="8"/>
     </row>
@@ -3158,17 +3167,17 @@
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
         <v>2026-03-11</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F29" s="8"/>
     </row>
@@ -3177,17 +3186,17 @@
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
         <v>2026-02-27</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F30" s="8"/>
     </row>
@@ -3196,17 +3205,17 @@
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
         <v>2026-03-10</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F31" s="8"/>
     </row>
@@ -3215,17 +3224,17 @@
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
         <v>2026-03-12</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F32" s="8"/>
     </row>
@@ -3234,17 +3243,17 @@
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
         <v>2026-02-11</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F33" s="8"/>
     </row>
@@ -3253,17 +3262,17 @@
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -3272,17 +3281,17 @@
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -3291,17 +3300,17 @@
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -3310,17 +3319,17 @@
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -3329,17 +3338,17 @@
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
         <v>2026-03-09</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -3348,17 +3357,17 @@
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
         <v>2026-02-12</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -3367,10 +3376,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3386,17 +3395,17 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
         <v>2026-02-07</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -3405,17 +3414,17 @@
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
         <v>2026-03-20 – 2026-03-21</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -3424,17 +3433,17 @@
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
         <v>2026-03-22</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -3459,12 +3468,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
@@ -3477,7 +3486,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
@@ -3485,16 +3494,16 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
@@ -3503,11 +3512,11 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3516,7 +3525,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
@@ -3528,16 +3537,16 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>

</xml_diff>

<commit_message>
Chap 5, EX 8
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35B6D921-4AD6-4932-811C-908664088637}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AC6605-80C7-4EEE-B04D-358301EC5CB7}"/>
   <bookViews>
     <workbookView xWindow="6015" yWindow="1830" windowWidth="22095" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="157">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -509,6 +509,10 @@
   </si>
   <si>
     <t>Actual done: 2026-02-06</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-08</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1180,7 +1184,9 @@
         <f t="shared" si="1"/>
         <v>46058</v>
       </c>
-      <c r="I8" s="8"/>
+      <c r="I8" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="J8" s="8" t="s">
         <v>24</v>
       </c>
@@ -1211,7 +1217,9 @@
         <f t="shared" si="1"/>
         <v>46059</v>
       </c>
-      <c r="I9" s="8"/>
+      <c r="I9" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="J9" s="8" t="s">
         <v>26</v>
       </c>
@@ -1364,14 +1372,16 @@
         <v>60</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H14" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46064</v>
       </c>
       <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
+      <c r="J14" s="13" t="s">
+        <v>156</v>
+      </c>
       <c r="K14" s="8"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.15">
@@ -3498,7 +3508,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3516,7 +3526,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3541,7 +3551,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
@@ -3550,12 +3560,12 @@
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, EX 13
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AC6605-80C7-4EEE-B04D-358301EC5CB7}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B501149E-0FEA-4A49-8391-3B874262A7C6}"/>
   <bookViews>
-    <workbookView xWindow="6015" yWindow="1830" windowWidth="22095" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3225" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="158">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -513,6 +513,10 @@
   </si>
   <si>
     <t>Actual done: 2026-02-08</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-09</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1403,14 +1407,16 @@
         <v>90</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H15" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46065</v>
       </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+      <c r="J15" s="13" t="s">
+        <v>157</v>
+      </c>
       <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.15">
@@ -3508,7 +3514,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3526,7 +3532,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3551,7 +3557,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 30
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_318C703A9E7610187CACADA6FFC7A1317313BD0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B501149E-0FEA-4A49-8391-3B874262A7C6}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3225" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="20490" windowHeight="7785"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -21,25 +15,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Plan'!$A$4:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercise Map'!$A$3:$F$43</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="159">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -125,39 +106,57 @@
     <t>Exercises: Ex6(a–c) (L1)</t>
   </si>
   <si>
+    <t>(a)(b): 2026-02-04, © 2026-02-05</t>
+  </si>
+  <si>
     <t>Exercises: Ex10 (L1) + 10-min recap note</t>
   </si>
   <si>
+    <t>Actual done: 2026-02-05</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>Read §5.3 (first half)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex38 (L2)</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-06</t>
+  </si>
+  <si>
+    <t>Read §5.3 (second half)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex7 (L2)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex8(a–b) (L3)</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-08</t>
+  </si>
+  <si>
+    <t>Exercises: Ex13 (L1)</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-09</t>
+  </si>
+  <si>
+    <t>Exercises: Ex30 (L1)</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-10</t>
+  </si>
+  <si>
+    <t>Exercises: Ex36 (L1)</t>
+  </si>
+  <si>
     <t>Not Started</t>
   </si>
   <si>
-    <t>5.3</t>
-  </si>
-  <si>
-    <t>Read §5.3 (first half)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex38 (L2)</t>
-  </si>
-  <si>
-    <t>Read §5.3 (second half)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex7 (L2)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex8(a–b) (L3)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex13 (L1)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex30 (L1)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex36 (L1)</t>
-  </si>
-  <si>
     <t>Exercises: Ex15(a–b) (L3) + quick §5.3 review</t>
   </si>
   <si>
@@ -498,36 +497,20 @@
   </si>
   <si>
     <t>C1 Marked Yes</t>
-  </si>
-  <si>
-    <t>Actual done: 2026-02-05</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>(a)(b): 2026-02-04, © 2026-02-05</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Actual done: 2026-02-06</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Actual done: 2026-02-08</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Actual done: 2026-02-09</t>
-    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,22 +544,158 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
-      <family val="3"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <family val="3"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -595,8 +714,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -619,11 +924,253 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -643,6 +1190,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -651,21 +1199,66 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -679,7 +1272,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -689,15 +1282,8 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -979,14 +1565,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1000,22 +1586,12 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" ht="20.25" spans="1:1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1029,46 +1605,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A4" s="9" t="s">
+    <row r="4" ht="27" spans="1:11">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A5" s="10">
+    <row r="5" spans="1:11">
+      <c r="A5" s="11">
         <v>1</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="12">
         <f t="shared" ref="B5:B36" si="0">IF($B$2="","",$B$2+A5-1)</f>
         <v>46053</v>
       </c>
@@ -1085,7 +1661,7 @@
       <c r="G5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f t="shared" ref="H5:H36" si="1">IF(G5="Done",B5+2,"")</f>
         <v>46055</v>
       </c>
@@ -1097,11 +1673,11 @@
       </c>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A6" s="10">
+    <row r="6" spans="1:11">
+      <c r="A6" s="11">
         <v>2</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="12">
         <f t="shared" si="0"/>
         <v>46054</v>
       </c>
@@ -1118,7 +1694,7 @@
       <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f t="shared" si="1"/>
         <v>46056</v>
       </c>
@@ -1130,11 +1706,11 @@
       </c>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A7" s="10">
+    <row r="7" spans="1:11">
+      <c r="A7" s="11">
         <v>3</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="12">
         <f t="shared" si="0"/>
         <v>46055</v>
       </c>
@@ -1151,7 +1727,7 @@
       <c r="G7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="13">
         <f t="shared" si="1"/>
         <v>46057</v>
       </c>
@@ -1163,11 +1739,11 @@
       </c>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A8" s="10">
+    <row r="8" spans="1:11">
+      <c r="A8" s="11">
         <v>4</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="12">
         <f t="shared" si="0"/>
         <v>46056</v>
       </c>
@@ -1184,7 +1760,7 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="13">
         <f t="shared" si="1"/>
         <v>46058</v>
       </c>
@@ -1196,11 +1772,11 @@
       </c>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A9" s="10">
+    <row r="9" spans="1:11">
+      <c r="A9" s="11">
         <v>5</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="12">
         <f t="shared" si="0"/>
         <v>46057</v>
       </c>
@@ -1217,7 +1793,7 @@
       <c r="G9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="13">
         <f t="shared" si="1"/>
         <v>46059</v>
       </c>
@@ -1229,11 +1805,11 @@
       </c>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A10" s="10">
+    <row r="10" ht="27" spans="1:11">
+      <c r="A10" s="11">
         <v>6</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="12">
         <f t="shared" si="0"/>
         <v>46058</v>
       </c>
@@ -1250,21 +1826,21 @@
       <c r="G10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="13">
         <f t="shared" si="1"/>
         <v>46060</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="13" t="s">
-        <v>154</v>
+      <c r="J10" s="14" t="s">
+        <v>28</v>
       </c>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A11" s="10">
+    <row r="11" spans="1:11">
+      <c r="A11" s="11">
         <v>7</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="12">
         <f t="shared" si="0"/>
         <v>46059</v>
       </c>
@@ -1273,7 +1849,7 @@
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" s="8">
         <v>60</v>
@@ -1281,32 +1857,32 @@
       <c r="G11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="13">
         <f t="shared" si="1"/>
         <v>46061</v>
       </c>
       <c r="I11" s="8"/>
-      <c r="J11" s="13" t="s">
-        <v>153</v>
+      <c r="J11" s="14" t="s">
+        <v>30</v>
       </c>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A12" s="10">
+    <row r="12" spans="1:11">
+      <c r="A12" s="11">
         <v>8</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="12">
         <f t="shared" si="0"/>
         <v>46060</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F12" s="8">
         <v>75</v>
@@ -1314,32 +1890,32 @@
       <c r="G12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="13">
         <f t="shared" si="1"/>
         <v>46062</v>
       </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="13" t="s">
-        <v>155</v>
+      <c r="J12" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="K12" s="8"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A13" s="10">
+    <row r="13" spans="1:11">
+      <c r="A13" s="11">
         <v>9</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="12">
         <f t="shared" si="0"/>
         <v>46061</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F13" s="8">
         <v>75</v>
@@ -1347,30 +1923,30 @@
       <c r="G13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="13">
         <f t="shared" si="1"/>
         <v>46063</v>
       </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="13" t="s">
-        <v>155</v>
+      <c r="J13" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A14" s="10">
+    <row r="14" spans="1:11">
+      <c r="A14" s="11">
         <v>10</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="12">
         <f t="shared" si="0"/>
         <v>46062</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F14" s="8">
         <v>60</v>
@@ -1378,30 +1954,30 @@
       <c r="G14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="13">
         <f t="shared" si="1"/>
         <v>46064</v>
       </c>
       <c r="I14" s="8"/>
-      <c r="J14" s="13" t="s">
-        <v>156</v>
+      <c r="J14" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A15" s="10">
+    <row r="15" spans="1:11">
+      <c r="A15" s="11">
         <v>11</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="12">
         <f t="shared" si="0"/>
         <v>46063</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F15" s="8">
         <v>90</v>
@@ -1409,67 +1985,69 @@
       <c r="G15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="13">
         <f t="shared" si="1"/>
         <v>46065</v>
       </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="13" t="s">
-        <v>157</v>
+      <c r="J15" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A16" s="10">
+    <row r="16" spans="1:11">
+      <c r="A16" s="11">
         <v>12</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="12">
         <f t="shared" si="0"/>
         <v>46064</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F16" s="8">
         <v>90</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H16" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H16" s="13">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46066</v>
       </c>
       <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+      <c r="J16" s="14" t="s">
+        <v>42</v>
+      </c>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A17" s="10">
+    <row r="17" spans="1:11">
+      <c r="A17" s="11">
         <v>13</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="12">
         <f t="shared" si="0"/>
         <v>46065</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="8" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F17" s="8">
         <v>90</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H17" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H17" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1477,28 +2055,28 @@
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A18" s="10">
+    <row r="18" ht="27" spans="1:11">
+      <c r="A18" s="11">
         <v>14</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="12">
         <f t="shared" si="0"/>
         <v>46066</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F18" s="8">
         <v>45</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H18" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H18" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1506,30 +2084,30 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A19" s="10">
+    <row r="19" spans="1:11">
+      <c r="A19" s="11">
         <v>15</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="12">
         <f t="shared" si="0"/>
         <v>46067</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F19" s="8">
         <v>75</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H19" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1537,28 +2115,28 @@
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A20" s="10">
+    <row r="20" spans="1:11">
+      <c r="A20" s="11">
         <v>16</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="12">
         <f t="shared" si="0"/>
         <v>46068</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F20" s="8">
         <v>60</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H20" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H20" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1566,30 +2144,30 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A21" s="10">
+    <row r="21" spans="1:11">
+      <c r="A21" s="11">
         <v>17</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="12">
         <f t="shared" si="0"/>
         <v>46069</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F21" s="8">
         <v>75</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H21" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H21" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1597,28 +2175,28 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A22" s="10">
+    <row r="22" spans="1:11">
+      <c r="A22" s="11">
         <v>18</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="12">
         <f t="shared" si="0"/>
         <v>46070</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="F22" s="8">
         <v>90</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H22" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H22" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1626,28 +2204,28 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A23" s="10">
+    <row r="23" spans="1:11">
+      <c r="A23" s="11">
         <v>19</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="12">
         <f t="shared" si="0"/>
         <v>46071</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="F23" s="8">
         <v>90</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H23" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H23" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1655,28 +2233,28 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A24" s="10">
+    <row r="24" spans="1:11">
+      <c r="A24" s="11">
         <v>20</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="12">
         <f t="shared" si="0"/>
         <v>46072</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F24" s="8">
         <v>90</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H24" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H24" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1684,28 +2262,28 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A25" s="10">
+    <row r="25" spans="1:11">
+      <c r="A25" s="11">
         <v>21</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="12">
         <f t="shared" si="0"/>
         <v>46073</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F25" s="8">
         <v>60</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H25" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H25" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1713,30 +2291,30 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A26" s="10">
+    <row r="26" spans="1:11">
+      <c r="A26" s="11">
         <v>22</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="12">
         <f t="shared" si="0"/>
         <v>46074</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F26" s="8">
         <v>75</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H26" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H26" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1744,28 +2322,28 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A27" s="10">
+    <row r="27" spans="1:11">
+      <c r="A27" s="11">
         <v>23</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="12">
         <f t="shared" si="0"/>
         <v>46075</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F27" s="8">
         <v>45</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H27" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H27" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1773,30 +2351,30 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A28" s="10">
+    <row r="28" spans="1:11">
+      <c r="A28" s="11">
         <v>24</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="12">
         <f t="shared" si="0"/>
         <v>46076</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F28" s="8">
         <v>75</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H28" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H28" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1804,28 +2382,28 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A29" s="10">
+    <row r="29" spans="1:11">
+      <c r="A29" s="11">
         <v>25</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="12">
         <f t="shared" si="0"/>
         <v>46077</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F29" s="8">
         <v>90</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H29" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H29" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1833,28 +2411,28 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A30" s="10">
+    <row r="30" spans="1:11">
+      <c r="A30" s="11">
         <v>26</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="12">
         <f t="shared" si="0"/>
         <v>46078</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F30" s="8">
         <v>90</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H30" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H30" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1862,28 +2440,28 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A31" s="10">
+    <row r="31" spans="1:11">
+      <c r="A31" s="11">
         <v>27</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="12">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F31" s="8">
         <v>75</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H31" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H31" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1891,28 +2469,28 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A32" s="10">
+    <row r="32" spans="1:11">
+      <c r="A32" s="11">
         <v>28</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="12">
         <f t="shared" si="0"/>
         <v>46080</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F32" s="8">
         <v>45</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H32" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H32" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1920,30 +2498,30 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A33" s="10">
+    <row r="33" spans="1:11">
+      <c r="A33" s="11">
         <v>29</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="12">
         <f t="shared" si="0"/>
         <v>46081</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F33" s="8">
         <v>75</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H33" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H33" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1951,28 +2529,28 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A34" s="10">
+    <row r="34" spans="1:11">
+      <c r="A34" s="11">
         <v>30</v>
       </c>
-      <c r="B34" s="11">
+      <c r="B34" s="12">
         <f t="shared" si="0"/>
         <v>46082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F34" s="8">
         <v>75</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H34" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H34" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -1980,28 +2558,28 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A35" s="10">
+    <row r="35" spans="1:11">
+      <c r="A35" s="11">
         <v>31</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="12">
         <f t="shared" si="0"/>
         <v>46083</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F35" s="8">
         <v>60</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H35" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H35" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2009,28 +2587,28 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A36" s="10">
+    <row r="36" spans="1:11">
+      <c r="A36" s="11">
         <v>32</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="12">
         <f t="shared" si="0"/>
         <v>46084</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F36" s="8">
         <v>90</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H36" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H36" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2038,30 +2616,30 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A37" s="10">
+    <row r="37" spans="1:11">
+      <c r="A37" s="11">
         <v>33</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="12">
         <f t="shared" ref="B37:B56" si="2">IF($B$2="","",$B$2+A37-1)</f>
         <v>46085</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F37" s="8">
         <v>90</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H37" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H37" s="13" t="str">
         <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
         <v/>
       </c>
@@ -2069,30 +2647,30 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A38" s="10">
+    <row r="38" spans="1:11">
+      <c r="A38" s="11">
         <v>34</v>
       </c>
-      <c r="B38" s="11">
+      <c r="B38" s="12">
         <f t="shared" si="2"/>
         <v>46086</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F38" s="8">
         <v>90</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H38" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H38" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2100,28 +2678,28 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A39" s="10">
+    <row r="39" spans="1:11">
+      <c r="A39" s="11">
         <v>35</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="12">
         <f t="shared" si="2"/>
         <v>46087</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F39" s="8">
         <v>60</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H39" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H39" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2129,28 +2707,28 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A40" s="10">
+    <row r="40" spans="1:11">
+      <c r="A40" s="11">
         <v>36</v>
       </c>
-      <c r="B40" s="11">
+      <c r="B40" s="12">
         <f t="shared" si="2"/>
         <v>46088</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F40" s="8">
         <v>90</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H40" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H40" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2158,28 +2736,28 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A41" s="10">
+    <row r="41" spans="1:11">
+      <c r="A41" s="11">
         <v>37</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="12">
         <f t="shared" si="2"/>
         <v>46089</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H41" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H41" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2187,28 +2765,28 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A42" s="10">
+    <row r="42" spans="1:11">
+      <c r="A42" s="11">
         <v>38</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="12">
         <f t="shared" si="2"/>
         <v>46090</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H42" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H42" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2216,28 +2794,28 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A43" s="10">
+    <row r="43" spans="1:11">
+      <c r="A43" s="11">
         <v>39</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="12">
         <f t="shared" si="2"/>
         <v>46091</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H43" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H43" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2245,28 +2823,28 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A44" s="10">
+    <row r="44" spans="1:11">
+      <c r="A44" s="11">
         <v>40</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="12">
         <f t="shared" si="2"/>
         <v>46092</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H44" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H44" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2274,28 +2852,28 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A45" s="10">
+    <row r="45" spans="1:11">
+      <c r="A45" s="11">
         <v>41</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="12">
         <f t="shared" si="2"/>
         <v>46093</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H45" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H45" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2303,28 +2881,28 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A46" s="10">
+    <row r="46" spans="1:11">
+      <c r="A46" s="11">
         <v>42</v>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="12">
         <f t="shared" si="2"/>
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H46" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H46" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2332,28 +2910,28 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A47" s="10">
+    <row r="47" spans="1:11">
+      <c r="A47" s="11">
         <v>43</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="12">
         <f t="shared" si="2"/>
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H47" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H47" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2361,28 +2939,28 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A48" s="10">
+    <row r="48" spans="1:11">
+      <c r="A48" s="11">
         <v>44</v>
       </c>
-      <c r="B48" s="11">
+      <c r="B48" s="12">
         <f t="shared" si="2"/>
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H48" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H48" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2390,28 +2968,28 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A49" s="10">
+    <row r="49" spans="1:11">
+      <c r="A49" s="11">
         <v>45</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="12">
         <f t="shared" si="2"/>
         <v>46097</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H49" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H49" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2419,28 +2997,28 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A50" s="10">
+    <row r="50" spans="1:11">
+      <c r="A50" s="11">
         <v>46</v>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="12">
         <f t="shared" si="2"/>
         <v>46098</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H50" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H50" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2448,11 +3026,11 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A51" s="10">
+    <row r="51" spans="1:11">
+      <c r="A51" s="11">
         <v>47</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="12">
         <f t="shared" si="2"/>
         <v>46099</v>
       </c>
@@ -2461,15 +3039,15 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H51" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H51" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2477,28 +3055,28 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A52" s="10">
+    <row r="52" spans="1:11">
+      <c r="A52" s="11">
         <v>48</v>
       </c>
-      <c r="B52" s="11">
+      <c r="B52" s="12">
         <f t="shared" si="2"/>
         <v>46100</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H52" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H52" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2506,28 +3084,28 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A53" s="10">
+    <row r="53" spans="1:11">
+      <c r="A53" s="11">
         <v>49</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="12">
         <f t="shared" si="2"/>
         <v>46101</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H53" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H53" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2535,28 +3113,28 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A54" s="10">
+    <row r="54" spans="1:11">
+      <c r="A54" s="11">
         <v>50</v>
       </c>
-      <c r="B54" s="11">
+      <c r="B54" s="12">
         <f t="shared" si="2"/>
         <v>46102</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H54" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H54" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2564,28 +3142,28 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A55" s="10">
+    <row r="55" spans="1:11">
+      <c r="A55" s="11">
         <v>51</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="12">
         <f t="shared" si="2"/>
         <v>46103</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H55" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H55" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2593,28 +3171,28 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A56" s="10">
+    <row r="56" ht="27" spans="1:11">
+      <c r="A56" s="11">
         <v>52</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="12">
         <f t="shared" si="2"/>
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H56" s="12" t="str">
+        <v>44</v>
+      </c>
+      <c r="H56" s="13" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2623,38 +3201,41 @@
       <c r="K56" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K56" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:K56">
+    <extLst/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A5:K56">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G5="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>$G5="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>$G5="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="G5:G56" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="G5:G56">
       <formula1>"Not Started,In Progress,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I5:I56" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I5:I56">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2664,54 +3245,49 @@
     <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="1" ht="18.75" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="3" ht="27" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6">
       <c r="A4" s="8">
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -2722,15 +3298,15 @@
       </c>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6">
       <c r="A5" s="8">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2741,15 +3317,15 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6">
       <c r="A6" s="8">
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -2760,15 +3336,15 @@
       </c>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6">
       <c r="A7" s="8">
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2779,15 +3355,15 @@
       </c>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="8" ht="27" spans="1:6">
       <c r="A8" s="8">
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -2798,91 +3374,91 @@
       </c>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="9" ht="27" spans="1:6">
       <c r="A9" s="8">
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:6">
       <c r="A10" s="8">
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
         <v>2026-02-08</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:6">
       <c r="A11" s="8">
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
         <v>2026-02-09</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:6">
       <c r="A12" s="8">
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
         <v>2026-03-19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:6">
       <c r="A13" s="8">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -2893,509 +3469,509 @@
       </c>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:6">
       <c r="A14" s="8">
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
         <v>2026-03-02</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="15" ht="27" spans="1:6">
       <c r="A15" s="8">
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
         <v>2026-02-24 – 2026-02-25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:6">
       <c r="A16" s="8">
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
         <v>2026-02-10</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:6">
       <c r="A17" s="8">
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
         <v>2026-02-16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:6">
       <c r="A18" s="8">
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
         <v>2026-02-13</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="19" ht="27" spans="1:6">
       <c r="A19" s="8">
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:6">
       <c r="A20" s="8">
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
         <v>2026-02-26</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:6">
       <c r="A21" s="8">
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
         <v>2026-02-22</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:6">
       <c r="A22" s="8">
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
         <v>2026-03-03</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="23" ht="27" spans="1:6">
       <c r="A23" s="8">
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
         <v>2026-02-17 – 2026-02-19</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:6">
       <c r="A24" s="8">
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
         <v>2026-02-20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="25" ht="27" spans="1:6">
       <c r="A25" s="8">
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
         <v>2026-03-04 – 2026-03-07</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:6">
       <c r="A26" s="8">
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
         <v>2026-02-23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:6">
       <c r="A27" s="8">
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
         <v>2026-03-08</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="28" ht="27" spans="1:6">
       <c r="A28" s="8">
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
         <v>2026-03-16 – 2026-03-17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:6">
       <c r="A29" s="8">
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
         <v>2026-03-11</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:6">
       <c r="A30" s="8">
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
         <v>2026-02-27</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:6">
       <c r="A31" s="8">
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
         <v>2026-03-10</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:6">
       <c r="A32" s="8">
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
         <v>2026-03-12</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:6">
       <c r="A33" s="8">
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
         <v>2026-02-11</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="34" ht="27" spans="1:6">
       <c r="A34" s="8">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:6">
       <c r="A35" s="8">
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F35" s="8"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:6">
       <c r="A36" s="8">
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F36" s="8"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:6">
       <c r="A37" s="8">
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:6">
       <c r="A38" s="8">
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
         <v>2026-03-09</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:6">
       <c r="A39" s="8">
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
         <v>2026-02-12</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:6">
       <c r="A40" s="8">
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3406,163 +3982,166 @@
       </c>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:6">
       <c r="A41" s="8">
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
         <v>2026-02-07</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F41" s="8"/>
     </row>
-    <row r="42" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="42" ht="27" spans="1:6">
       <c r="A42" s="8">
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
         <v>2026-03-20 – 2026-03-21</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F42" s="8"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:6">
       <c r="A43" s="8">
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
         <v>2026-03-22</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F43" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F43" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:F43">
+    <extLst/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:2">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
@@ -3570,8 +4149,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, EX 36, modified EX 8(a)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F572FC63-E749-4F92-B03E-22845E3CE877}"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7785"/>
+    <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -15,12 +21,25 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Plan'!$A$4:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercise Map'!$A$3:$F$43</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="162">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -169,6 +188,12 @@
     <t>Exercises: Ex6(d) (L1)</t>
   </si>
   <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Read 5.4 at 2026-02-10</t>
+  </si>
+  <si>
     <t>Exercises: Ex6(e) (L1) (finish Ex6)</t>
   </si>
   <si>
@@ -497,20 +522,20 @@
   </si>
   <si>
     <t>C1 Marked Yes</t>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-11</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -544,158 +569,22 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="9"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -714,194 +603,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -924,253 +627,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="20" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1190,7 +651,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1199,66 +659,21 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1272,7 +687,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1282,8 +697,15 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1565,14 +987,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1586,12 +1008,22 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" spans="1:1">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1605,46 +1037,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="27" spans="1:11">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="11">
         <f t="shared" ref="B5:B36" si="0">IF($B$2="","",$B$2+A5-1)</f>
         <v>46053</v>
       </c>
@@ -1661,7 +1093,7 @@
       <c r="G5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="12">
         <f t="shared" ref="H5:H36" si="1">IF(G5="Done",B5+2,"")</f>
         <v>46055</v>
       </c>
@@ -1673,11 +1105,11 @@
       </c>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A6" s="10">
         <v>2</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>46054</v>
       </c>
@@ -1694,7 +1126,7 @@
       <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="12">
         <f t="shared" si="1"/>
         <v>46056</v>
       </c>
@@ -1706,11 +1138,11 @@
       </c>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A7" s="10">
         <v>3</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="11">
         <f t="shared" si="0"/>
         <v>46055</v>
       </c>
@@ -1727,7 +1159,7 @@
       <c r="G7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <f t="shared" si="1"/>
         <v>46057</v>
       </c>
@@ -1739,11 +1171,11 @@
       </c>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A8" s="10">
         <v>4</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>46056</v>
       </c>
@@ -1760,7 +1192,7 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="12">
         <f t="shared" si="1"/>
         <v>46058</v>
       </c>
@@ -1772,11 +1204,11 @@
       </c>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A9" s="10">
         <v>5</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="11">
         <f t="shared" si="0"/>
         <v>46057</v>
       </c>
@@ -1793,7 +1225,7 @@
       <c r="G9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <f t="shared" si="1"/>
         <v>46059</v>
       </c>
@@ -1805,11 +1237,11 @@
       </c>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" ht="27" spans="1:11">
-      <c r="A10" s="11">
+    <row r="10" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A10" s="10">
         <v>6</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>46058</v>
       </c>
@@ -1826,21 +1258,21 @@
       <c r="G10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="12">
         <f t="shared" si="1"/>
         <v>46060</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A11" s="10">
         <v>7</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="11">
         <f t="shared" si="0"/>
         <v>46059</v>
       </c>
@@ -1857,21 +1289,21 @@
       <c r="G11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="12">
         <f t="shared" si="1"/>
         <v>46061</v>
       </c>
       <c r="I11" s="8"/>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A12" s="10">
         <v>8</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>46060</v>
       </c>
@@ -1890,21 +1322,21 @@
       <c r="G12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <f t="shared" si="1"/>
         <v>46062</v>
       </c>
       <c r="I12" s="8"/>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="8" t="s">
         <v>34</v>
       </c>
       <c r="K12" s="8"/>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A13" s="10">
         <v>9</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="11">
         <f t="shared" si="0"/>
         <v>46061</v>
       </c>
@@ -1923,21 +1355,21 @@
       <c r="G13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="13">
+      <c r="H13" s="12">
         <f t="shared" si="1"/>
         <v>46063</v>
       </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="14" t="s">
+      <c r="J13" s="8" t="s">
         <v>34</v>
       </c>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A14" s="10">
         <v>10</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>46062</v>
       </c>
@@ -1954,21 +1386,21 @@
       <c r="G14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="13">
+      <c r="H14" s="12">
         <f t="shared" si="1"/>
         <v>46064</v>
       </c>
       <c r="I14" s="8"/>
-      <c r="J14" s="14" t="s">
+      <c r="J14" s="8" t="s">
         <v>38</v>
       </c>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A15" s="10">
         <v>11</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <f t="shared" si="0"/>
         <v>46063</v>
       </c>
@@ -1985,21 +1417,23 @@
       <c r="G15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="13">
+      <c r="H15" s="12">
         <f t="shared" si="1"/>
         <v>46065</v>
       </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="14" t="s">
+      <c r="I15" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>40</v>
       </c>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A16" s="10">
         <v>12</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>46064</v>
       </c>
@@ -2016,21 +1450,23 @@
       <c r="G16" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="13">
+      <c r="H16" s="12">
         <f t="shared" si="1"/>
         <v>46066</v>
       </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="14" t="s">
+      <c r="I16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>42</v>
       </c>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A17" s="10">
         <v>13</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="11">
         <f t="shared" si="0"/>
         <v>46065</v>
       </c>
@@ -2045,21 +1481,23 @@
         <v>90</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H17" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H17" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46067</v>
       </c>
       <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+      <c r="J17" s="13" t="s">
+        <v>161</v>
+      </c>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" ht="27" spans="1:11">
-      <c r="A18" s="11">
+    <row r="18" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A18" s="10">
         <v>14</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <f t="shared" si="0"/>
         <v>46066</v>
       </c>
@@ -2076,7 +1514,7 @@
       <c r="G18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="13" t="str">
+      <c r="H18" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2084,11 +1522,11 @@
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A19" s="10">
         <v>15</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="11">
         <f t="shared" si="0"/>
         <v>46067</v>
       </c>
@@ -2105,21 +1543,23 @@
         <v>75</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H19" s="13" t="str">
+        <v>49</v>
+      </c>
+      <c r="H19" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="J19" s="8" t="s">
+        <v>50</v>
+      </c>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A20" s="10">
         <v>16</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>46068</v>
       </c>
@@ -2128,7 +1568,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F20" s="8">
         <v>60</v>
@@ -2136,7 +1576,7 @@
       <c r="G20" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H20" s="13" t="str">
+      <c r="H20" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2144,22 +1584,22 @@
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A21" s="10">
         <v>17</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="11">
         <f t="shared" si="0"/>
         <v>46069</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F21" s="8">
         <v>75</v>
@@ -2167,7 +1607,7 @@
       <c r="G21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H21" s="13" t="str">
+      <c r="H21" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2175,20 +1615,20 @@
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A22" s="10">
         <v>18</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>46070</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F22" s="8">
         <v>90</v>
@@ -2196,7 +1636,7 @@
       <c r="G22" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H22" s="13" t="str">
+      <c r="H22" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2204,20 +1644,20 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A23" s="10">
         <v>19</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="11">
         <f t="shared" si="0"/>
         <v>46071</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F23" s="8">
         <v>90</v>
@@ -2225,7 +1665,7 @@
       <c r="G23" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H23" s="13" t="str">
+      <c r="H23" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2233,20 +1673,20 @@
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A24" s="10">
         <v>20</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="11">
         <f t="shared" si="0"/>
         <v>46072</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F24" s="8">
         <v>90</v>
@@ -2254,7 +1694,7 @@
       <c r="G24" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="13" t="str">
+      <c r="H24" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2262,20 +1702,20 @@
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A25" s="10">
         <v>21</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="11">
         <f t="shared" si="0"/>
         <v>46073</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F25" s="8">
         <v>60</v>
@@ -2283,7 +1723,7 @@
       <c r="G25" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="13" t="str">
+      <c r="H25" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2291,22 +1731,22 @@
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A26" s="10">
         <v>22</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>46074</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F26" s="8">
         <v>75</v>
@@ -2314,7 +1754,7 @@
       <c r="G26" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H26" s="13" t="str">
+      <c r="H26" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2322,20 +1762,20 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A27" s="10">
         <v>23</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="11">
         <f t="shared" si="0"/>
         <v>46075</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F27" s="8">
         <v>45</v>
@@ -2343,7 +1783,7 @@
       <c r="G27" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H27" s="13" t="str">
+      <c r="H27" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2351,22 +1791,22 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A28" s="10">
         <v>24</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>46076</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F28" s="8">
         <v>75</v>
@@ -2374,7 +1814,7 @@
       <c r="G28" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="13" t="str">
+      <c r="H28" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2382,20 +1822,20 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A29" s="10">
         <v>25</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="11">
         <f t="shared" si="0"/>
         <v>46077</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F29" s="8">
         <v>90</v>
@@ -2403,7 +1843,7 @@
       <c r="G29" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="13" t="str">
+      <c r="H29" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2411,20 +1851,20 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A30" s="10">
         <v>26</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>46078</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F30" s="8">
         <v>90</v>
@@ -2432,7 +1872,7 @@
       <c r="G30" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H30" s="13" t="str">
+      <c r="H30" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2440,20 +1880,20 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A31" s="10">
         <v>27</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="11">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F31" s="8">
         <v>75</v>
@@ -2461,7 +1901,7 @@
       <c r="G31" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H31" s="13" t="str">
+      <c r="H31" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2469,20 +1909,20 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A32" s="10">
         <v>28</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>46080</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F32" s="8">
         <v>45</v>
@@ -2490,7 +1930,7 @@
       <c r="G32" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H32" s="13" t="str">
+      <c r="H32" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2498,22 +1938,22 @@
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A33" s="10">
         <v>29</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="11">
         <f t="shared" si="0"/>
         <v>46081</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F33" s="8">
         <v>75</v>
@@ -2521,7 +1961,7 @@
       <c r="G33" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H33" s="13" t="str">
+      <c r="H33" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2529,20 +1969,20 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A34" s="10">
         <v>30</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>46082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F34" s="8">
         <v>75</v>
@@ -2550,7 +1990,7 @@
       <c r="G34" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H34" s="13" t="str">
+      <c r="H34" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2558,20 +1998,20 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A35" s="10">
         <v>31</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="11">
         <f t="shared" si="0"/>
         <v>46083</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F35" s="8">
         <v>60</v>
@@ -2579,7 +2019,7 @@
       <c r="G35" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H35" s="13" t="str">
+      <c r="H35" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2587,20 +2027,20 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A36" s="10">
         <v>32</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="11">
         <f t="shared" si="0"/>
         <v>46084</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F36" s="8">
         <v>90</v>
@@ -2608,7 +2048,7 @@
       <c r="G36" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="13" t="str">
+      <c r="H36" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -2616,22 +2056,22 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A37" s="10">
         <v>33</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="11">
         <f t="shared" ref="B37:B56" si="2">IF($B$2="","",$B$2+A37-1)</f>
         <v>46085</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F37" s="8">
         <v>90</v>
@@ -2639,7 +2079,7 @@
       <c r="G37" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H37" s="13" t="str">
+      <c r="H37" s="12" t="str">
         <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
         <v/>
       </c>
@@ -2647,22 +2087,22 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A38" s="10">
         <v>34</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="11">
         <f t="shared" si="2"/>
         <v>46086</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F38" s="8">
         <v>90</v>
@@ -2670,7 +2110,7 @@
       <c r="G38" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="13" t="str">
+      <c r="H38" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2678,20 +2118,20 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A39" s="10">
         <v>35</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="11">
         <f t="shared" si="2"/>
         <v>46087</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F39" s="8">
         <v>60</v>
@@ -2699,7 +2139,7 @@
       <c r="G39" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H39" s="13" t="str">
+      <c r="H39" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2707,20 +2147,20 @@
       <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11">
-      <c r="A40" s="11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A40" s="10">
         <v>36</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="11">
         <f t="shared" si="2"/>
         <v>46088</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F40" s="8">
         <v>90</v>
@@ -2728,7 +2168,7 @@
       <c r="G40" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H40" s="13" t="str">
+      <c r="H40" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2736,11 +2176,11 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A41" s="10">
         <v>37</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="11">
         <f t="shared" si="2"/>
         <v>46089</v>
       </c>
@@ -2749,7 +2189,7 @@
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
@@ -2757,7 +2197,7 @@
       <c r="G41" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H41" s="13" t="str">
+      <c r="H41" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2765,20 +2205,20 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11">
-      <c r="A42" s="11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A42" s="10">
         <v>38</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="11">
         <f t="shared" si="2"/>
         <v>46090</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
@@ -2786,7 +2226,7 @@
       <c r="G42" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H42" s="13" t="str">
+      <c r="H42" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2794,11 +2234,11 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11">
-      <c r="A43" s="11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A43" s="10">
         <v>39</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="11">
         <f t="shared" si="2"/>
         <v>46091</v>
       </c>
@@ -2807,7 +2247,7 @@
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
@@ -2815,7 +2255,7 @@
       <c r="G43" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="13" t="str">
+      <c r="H43" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2823,20 +2263,20 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11">
-      <c r="A44" s="11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A44" s="10">
         <v>40</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="11">
         <f t="shared" si="2"/>
         <v>46092</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
@@ -2844,7 +2284,7 @@
       <c r="G44" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H44" s="13" t="str">
+      <c r="H44" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2852,11 +2292,11 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A45" s="10">
         <v>41</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="11">
         <f t="shared" si="2"/>
         <v>46093</v>
       </c>
@@ -2865,7 +2305,7 @@
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
@@ -2873,7 +2313,7 @@
       <c r="G45" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H45" s="13" t="str">
+      <c r="H45" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2881,20 +2321,20 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A46" s="10">
         <v>42</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="11">
         <f t="shared" si="2"/>
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
@@ -2902,7 +2342,7 @@
       <c r="G46" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H46" s="13" t="str">
+      <c r="H46" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2910,20 +2350,20 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11">
-      <c r="A47" s="11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A47" s="10">
         <v>43</v>
       </c>
-      <c r="B47" s="12">
+      <c r="B47" s="11">
         <f t="shared" si="2"/>
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
@@ -2931,7 +2371,7 @@
       <c r="G47" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H47" s="13" t="str">
+      <c r="H47" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2939,20 +2379,20 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11">
-      <c r="A48" s="11">
-        <v>44</v>
-      </c>
-      <c r="B48" s="12">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A48" s="10">
+        <v>44</v>
+      </c>
+      <c r="B48" s="11">
         <f t="shared" si="2"/>
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
@@ -2960,7 +2400,7 @@
       <c r="G48" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H48" s="13" t="str">
+      <c r="H48" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2968,20 +2408,20 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11">
-      <c r="A49" s="11">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A49" s="10">
         <v>45</v>
       </c>
-      <c r="B49" s="12">
+      <c r="B49" s="11">
         <f t="shared" si="2"/>
         <v>46097</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
@@ -2989,7 +2429,7 @@
       <c r="G49" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H49" s="13" t="str">
+      <c r="H49" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2997,20 +2437,20 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11">
-      <c r="A50" s="11">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A50" s="10">
         <v>46</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="11">
         <f t="shared" si="2"/>
         <v>46098</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
@@ -3018,7 +2458,7 @@
       <c r="G50" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H50" s="13" t="str">
+      <c r="H50" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3026,11 +2466,11 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11">
-      <c r="A51" s="11">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A51" s="10">
         <v>47</v>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="11">
         <f t="shared" si="2"/>
         <v>46099</v>
       </c>
@@ -3039,7 +2479,7 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
@@ -3047,7 +2487,7 @@
       <c r="G51" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H51" s="13" t="str">
+      <c r="H51" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3055,20 +2495,20 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11">
-      <c r="A52" s="11">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A52" s="10">
         <v>48</v>
       </c>
-      <c r="B52" s="12">
+      <c r="B52" s="11">
         <f t="shared" si="2"/>
         <v>46100</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
@@ -3076,7 +2516,7 @@
       <c r="G52" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H52" s="13" t="str">
+      <c r="H52" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3084,20 +2524,20 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11">
-      <c r="A53" s="11">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A53" s="10">
         <v>49</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="11">
         <f t="shared" si="2"/>
         <v>46101</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
@@ -3105,7 +2545,7 @@
       <c r="G53" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H53" s="13" t="str">
+      <c r="H53" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3113,20 +2553,20 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11">
-      <c r="A54" s="11">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A54" s="10">
         <v>50</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="11">
         <f t="shared" si="2"/>
         <v>46102</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
@@ -3134,7 +2574,7 @@
       <c r="G54" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H54" s="13" t="str">
+      <c r="H54" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3142,20 +2582,20 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="11">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.15">
+      <c r="A55" s="10">
         <v>51</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="11">
         <f t="shared" si="2"/>
         <v>46103</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
@@ -3163,7 +2603,7 @@
       <c r="G55" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H55" s="13" t="str">
+      <c r="H55" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3171,20 +2611,20 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" ht="27" spans="1:11">
-      <c r="A56" s="11">
+    <row r="56" spans="1:11" ht="27" x14ac:dyDescent="0.15">
+      <c r="A56" s="10">
         <v>52</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="11">
         <f t="shared" si="2"/>
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
@@ -3192,7 +2632,7 @@
       <c r="G56" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H56" s="13" t="str">
+      <c r="H56" s="12" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -3201,41 +2641,38 @@
       <c r="K56" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K56">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A4:K56" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A5:K56">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$G5="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>$G5="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$G5="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="G5:G56">
+    <dataValidation type="list" sqref="G5:G56" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I5:I56">
+    <dataValidation type="list" allowBlank="1" sqref="I5:I56" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -3245,49 +2682,54 @@
     <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="3" ht="27" spans="1:6">
+    <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A4" s="8">
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -3298,15 +2740,15 @@
       </c>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A5" s="8">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3317,15 +2759,15 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A6" s="8">
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -3336,15 +2778,15 @@
       </c>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A7" s="8">
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3355,15 +2797,15 @@
       </c>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" ht="27" spans="1:6">
+    <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A8" s="8">
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -3374,34 +2816,34 @@
       </c>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" ht="27" spans="1:6">
+    <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A9" s="8">
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A10" s="8">
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -3412,15 +2854,15 @@
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A11" s="8">
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -3431,34 +2873,34 @@
       </c>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A12" s="8">
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
         <v>2026-03-19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A13" s="8">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3469,53 +2911,53 @@
       </c>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A14" s="8">
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
         <v>2026-03-02</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" ht="27" spans="1:6">
+    <row r="15" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A15" s="8">
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
         <v>2026-02-24 – 2026-02-25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A16" s="8">
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -3526,34 +2968,34 @@
       </c>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A17" s="8">
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
         <v>2026-02-16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A18" s="8">
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3564,167 +3006,167 @@
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" ht="27" spans="1:6">
+    <row r="19" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A19" s="8">
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A20" s="8">
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
         <v>2026-02-26</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A21" s="8">
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
         <v>2026-02-22</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A22" s="8">
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
         <v>2026-03-03</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" ht="27" spans="1:6">
+    <row r="23" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A23" s="8">
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
         <v>2026-02-17 – 2026-02-19</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A24" s="8">
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
         <v>2026-02-20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" ht="27" spans="1:6">
+    <row r="25" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A25" s="8">
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
         <v>2026-03-04 – 2026-03-07</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A26" s="8">
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
         <v>2026-02-23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A27" s="8">
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3735,72 +3177,72 @@
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" ht="27" spans="1:6">
+    <row r="28" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A28" s="8">
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
         <v>2026-03-16 – 2026-03-17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A29" s="8">
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
         <v>2026-03-11</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A30" s="8">
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
         <v>2026-02-27</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A31" s="8">
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3811,15 +3253,15 @@
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A32" s="8">
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3830,15 +3272,15 @@
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A33" s="8">
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3849,110 +3291,110 @@
       </c>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" ht="27" spans="1:6">
+    <row r="34" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A34" s="8">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A35" s="8">
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F35" s="8"/>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A36" s="8">
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F36" s="8"/>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A37" s="8">
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A38" s="8">
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
         <v>2026-03-09</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A39" s="8">
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -3963,15 +3405,15 @@
       </c>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" s="8">
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3982,15 +3424,15 @@
       </c>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A41" s="8">
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -4001,156 +3443,153 @@
       </c>
       <c r="F41" s="8"/>
     </row>
-    <row r="42" ht="27" spans="1:6">
+    <row r="42" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A42" s="8">
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
         <v>2026-03-20 – 2026-03-21</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F42" s="8"/>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A43" s="8">
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
         <v>2026-03-22</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F43" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F43">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A3:F43" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:1">
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, EX 6(d-e)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34E6B3B7-3E96-480F-9238-1EF5B3687A30}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7136A1CF-7550-40F6-A336-97A6DC62A1F0}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="164">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -188,9 +188,6 @@
     <t>Exercises: Ex6(d) (L1)</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>Read 5.4 at 2026-02-10</t>
   </si>
   <si>
@@ -525,6 +522,19 @@
   </si>
   <si>
     <t>Actual done: 2026-02-11</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-12</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-13</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Read 5.5 at 2026-02-12 
+Actual done: 2026-02-13</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1489,7 +1499,7 @@
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K17" s="8"/>
     </row>
@@ -1512,14 +1522,16 @@
         <v>45</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H18" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H18" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46068</v>
       </c>
       <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="J18" s="13" t="s">
+        <v>161</v>
+      </c>
       <c r="K18" s="8"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.15">
@@ -1543,15 +1555,15 @@
         <v>75</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H19" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H19" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46069</v>
       </c>
       <c r="I19" s="8"/>
       <c r="J19" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K19" s="8"/>
     </row>
@@ -1568,23 +1580,25 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F20" s="8">
         <v>60</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H20" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46070</v>
       </c>
       <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="J20" s="13" t="s">
+        <v>162</v>
+      </c>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:11" ht="27" x14ac:dyDescent="0.15">
       <c r="A21" s="10">
         <v>17</v>
       </c>
@@ -1593,26 +1607,28 @@
         <v>46069</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="F21" s="8">
         <v>75</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H21" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H21" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46071</v>
       </c>
       <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="J21" s="13" t="s">
+        <v>163</v>
+      </c>
       <c r="K21" s="8"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.15">
@@ -1624,11 +1640,11 @@
         <v>46070</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F22" s="8">
         <v>90</v>
@@ -1653,11 +1669,11 @@
         <v>46071</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F23" s="8">
         <v>90</v>
@@ -1682,11 +1698,11 @@
         <v>46072</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F24" s="8">
         <v>90</v>
@@ -1711,11 +1727,11 @@
         <v>46073</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F25" s="8">
         <v>60</v>
@@ -1740,13 +1756,13 @@
         <v>46074</v>
       </c>
       <c r="C26" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="8" t="s">
         <v>61</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>62</v>
       </c>
       <c r="F26" s="8">
         <v>75</v>
@@ -1771,11 +1787,11 @@
         <v>46075</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F27" s="8">
         <v>45</v>
@@ -1800,13 +1816,13 @@
         <v>46076</v>
       </c>
       <c r="C28" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="E28" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>66</v>
       </c>
       <c r="F28" s="8">
         <v>75</v>
@@ -1831,11 +1847,11 @@
         <v>46077</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F29" s="8">
         <v>90</v>
@@ -1860,11 +1876,11 @@
         <v>46078</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F30" s="8">
         <v>90</v>
@@ -1889,11 +1905,11 @@
         <v>46079</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F31" s="8">
         <v>75</v>
@@ -1918,11 +1934,11 @@
         <v>46080</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F32" s="8">
         <v>45</v>
@@ -1947,13 +1963,13 @@
         <v>46081</v>
       </c>
       <c r="C33" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>75</v>
       </c>
       <c r="F33" s="8">
         <v>75</v>
@@ -1978,11 +1994,11 @@
         <v>46082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F34" s="8">
         <v>75</v>
@@ -2007,11 +2023,11 @@
         <v>46083</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F35" s="8">
         <v>60</v>
@@ -2036,11 +2052,11 @@
         <v>46084</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F36" s="8">
         <v>90</v>
@@ -2065,13 +2081,13 @@
         <v>46085</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D37" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>81</v>
       </c>
       <c r="F37" s="8">
         <v>90</v>
@@ -2096,13 +2112,13 @@
         <v>46086</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D38" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="F38" s="8">
         <v>90</v>
@@ -2127,11 +2143,11 @@
         <v>46087</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F39" s="8">
         <v>60</v>
@@ -2156,11 +2172,11 @@
         <v>46088</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F40" s="8">
         <v>90</v>
@@ -2189,7 +2205,7 @@
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
@@ -2214,11 +2230,11 @@
         <v>46090</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
@@ -2247,7 +2263,7 @@
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
@@ -2272,11 +2288,11 @@
         <v>46092</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
@@ -2305,7 +2321,7 @@
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
@@ -2330,11 +2346,11 @@
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
@@ -2359,11 +2375,11 @@
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
@@ -2388,11 +2404,11 @@
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
@@ -2417,11 +2433,11 @@
         <v>46097</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
@@ -2446,11 +2462,11 @@
         <v>46098</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
@@ -2479,7 +2495,7 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
@@ -2504,11 +2520,11 @@
         <v>46100</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
@@ -2533,11 +2549,11 @@
         <v>46101</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
@@ -2562,11 +2578,11 @@
         <v>46102</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
@@ -2591,11 +2607,11 @@
         <v>46103</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
@@ -2620,11 +2636,11 @@
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
@@ -2684,7 +2700,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2694,7 +2710,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
@@ -2703,19 +2719,19 @@
     </row>
     <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>108</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>109</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
@@ -2726,10 +2742,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>111</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -2745,10 +2761,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2764,10 +2780,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -2783,10 +2799,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2802,10 +2818,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -2821,17 +2837,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -2840,10 +2856,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -2859,10 +2875,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -2878,17 +2894,17 @@
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
         <v>2026-03-19</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F12" s="8"/>
     </row>
@@ -2897,10 +2913,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>120</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>121</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -2916,17 +2932,17 @@
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
         <v>2026-03-02</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F14" s="8"/>
     </row>
@@ -2935,17 +2951,17 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
         <v>2026-02-24 – 2026-02-25</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -2954,10 +2970,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -2973,17 +2989,17 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
         <v>2026-02-16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F17" s="8"/>
     </row>
@@ -2992,10 +3008,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3011,17 +3027,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -3030,17 +3046,17 @@
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
         <v>2026-02-26</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -3049,17 +3065,17 @@
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>131</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
         <v>2026-02-22</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F21" s="8"/>
     </row>
@@ -3068,17 +3084,17 @@
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
         <v>2026-03-03</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F22" s="8"/>
     </row>
@@ -3087,17 +3103,17 @@
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
         <v>2026-02-17 – 2026-02-19</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F23" s="8"/>
     </row>
@@ -3106,17 +3122,17 @@
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
         <v>2026-02-20</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F24" s="8"/>
     </row>
@@ -3125,17 +3141,17 @@
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
         <v>2026-03-04 – 2026-03-07</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F25" s="8"/>
     </row>
@@ -3144,17 +3160,17 @@
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
         <v>2026-02-23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F26" s="8"/>
     </row>
@@ -3163,10 +3179,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3182,17 +3198,17 @@
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
         <v>2026-03-16 – 2026-03-17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F28" s="8"/>
     </row>
@@ -3201,17 +3217,17 @@
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
         <v>2026-03-11</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F29" s="8"/>
     </row>
@@ -3220,17 +3236,17 @@
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
         <v>2026-02-27</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F30" s="8"/>
     </row>
@@ -3239,10 +3255,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3258,10 +3274,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3277,10 +3293,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3296,17 +3312,17 @@
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -3315,17 +3331,17 @@
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -3334,17 +3350,17 @@
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -3353,17 +3369,17 @@
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -3372,17 +3388,17 @@
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
         <v>2026-03-09</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -3391,10 +3407,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -3410,10 +3426,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3429,10 +3445,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -3448,17 +3464,17 @@
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
         <v>2026-03-20 – 2026-03-21</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F42" s="8"/>
     </row>
@@ -3467,17 +3483,17 @@
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
         <v>2026-03-22</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F43" s="8"/>
     </row>
@@ -3502,12 +3518,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
@@ -3520,7 +3536,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
@@ -3528,29 +3544,29 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3559,7 +3575,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
@@ -3571,16 +3587,16 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
@@ -3590,6 +3606,6 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chap 5, summary 5.4-5.6, EX 20(a)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7136A1CF-7550-40F6-A336-97A6DC62A1F0}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8D100FE-6399-4925-A899-65D1CDA71C31}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="165">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -535,6 +535,10 @@
   <si>
     <t>Read 5.5 at 2026-02-12 
 Actual done: 2026-02-13</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-14</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1650,14 +1654,16 @@
         <v>90</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H22" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H22" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46072</v>
       </c>
       <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="J22" s="13" t="s">
+        <v>164</v>
+      </c>
       <c r="K22" s="8"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.15">
@@ -3548,7 +3554,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3566,7 +3572,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3591,7 +3597,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 21
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8D100FE-6399-4925-A899-65D1CDA71C31}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDF1EC55-755C-4038-809F-8929332DCAE1}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="168">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -539,6 +539,18 @@
   </si>
   <si>
     <t>Actual done: 2026-02-14</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-16</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-15</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-18</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1685,14 +1697,16 @@
         <v>90</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H23" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H23" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46073</v>
       </c>
       <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="J23" s="13" t="s">
+        <v>166</v>
+      </c>
       <c r="K23" s="8"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.15">
@@ -1714,14 +1728,16 @@
         <v>90</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H24" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H24" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46074</v>
       </c>
       <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
+      <c r="J24" s="13" t="s">
+        <v>165</v>
+      </c>
       <c r="K24" s="8"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.15">
@@ -1743,14 +1759,16 @@
         <v>60</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H25" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H25" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46075</v>
       </c>
       <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
+      <c r="J25" s="13" t="s">
+        <v>167</v>
+      </c>
       <c r="K25" s="8"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.15">
@@ -3554,7 +3572,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3572,7 +3590,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3597,7 +3615,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 16(a), 18
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDF1EC55-755C-4038-809F-8929332DCAE1}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68CC12ED-C74A-4A57-86F6-330435E4871D}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="169">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -551,6 +551,10 @@
   </si>
   <si>
     <t>Actual done: 2026-02-18</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-22</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1792,14 +1796,16 @@
         <v>75</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H26" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H26" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46076</v>
       </c>
       <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
+      <c r="J26" s="13" t="s">
+        <v>168</v>
+      </c>
       <c r="K26" s="8"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.15">
@@ -3572,7 +3578,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3590,7 +3596,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3615,7 +3621,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 23
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68CC12ED-C74A-4A57-86F6-330435E4871D}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A23A8A9-F292-4B82-8278-D1A8FA90803A}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="171">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -555,6 +555,14 @@
   </si>
   <si>
     <t>Actual done: 2026-02-22</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-02-25</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-03-01</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1827,14 +1835,16 @@
         <v>45</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H27" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H27" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46077</v>
       </c>
       <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
+      <c r="J27" s="13" t="s">
+        <v>169</v>
+      </c>
       <c r="K27" s="8"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.15">
@@ -1858,14 +1868,16 @@
         <v>75</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H28" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H28" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46078</v>
       </c>
       <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
+      <c r="J28" s="13" t="s">
+        <v>170</v>
+      </c>
       <c r="K28" s="8"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.15">
@@ -3578,7 +3590,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3596,7 +3608,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3621,7 +3633,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 12
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A23A8A9-F292-4B82-8278-D1A8FA90803A}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CEB0DC2-145D-4F3B-A09B-C48A398E4D9C}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="172">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -563,6 +563,10 @@
   </si>
   <si>
     <t>Actual done: 2026-03-01</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-03-04</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1899,11 +1903,11 @@
         <v>90</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H29" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H29" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46079</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
@@ -1928,14 +1932,16 @@
         <v>90</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H30" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H30" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46080</v>
       </c>
       <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
+      <c r="J30" s="13" t="s">
+        <v>171</v>
+      </c>
       <c r="K30" s="8"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.15">
@@ -3590,7 +3596,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3608,7 +3614,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3633,7 +3639,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 17
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CEB0DC2-145D-4F3B-A09B-C48A398E4D9C}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B110FBF-8BFB-4CCA-AFBE-1777FBA6ACB1}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="173">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -567,6 +567,10 @@
   </si>
   <si>
     <t>Actual done: 2026-03-04</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-03-06</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1963,14 +1967,16 @@
         <v>75</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H31" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H31" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46081</v>
       </c>
       <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
+      <c r="J31" s="13" t="s">
+        <v>172</v>
+      </c>
       <c r="K31" s="8"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.15">
@@ -3596,7 +3602,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3614,7 +3620,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3639,7 +3645,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 27
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B110FBF-8BFB-4CCA-AFBE-1777FBA6ACB1}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_0473CADABC03135558BEBFE63FE93A2CB1474B28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BCD6FDE-E80A-4BE6-9E07-769898D4E23D}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="174">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -571,6 +571,10 @@
   </si>
   <si>
     <t>Actual done: 2026-03-06</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual done: 2026-03-08</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1998,14 +2002,16 @@
         <v>45</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H32" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H32" s="12">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46082</v>
       </c>
       <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
+      <c r="J32" s="13" t="s">
+        <v>173</v>
+      </c>
       <c r="K32" s="8"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.15">
@@ -3602,7 +3608,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.15">
@@ -3620,7 +3626,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.15">
@@ -3645,7 +3651,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
Chap 5, EX 22(a)(b)(c)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="178">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -308,25 +308,28 @@
     <t>Exercises: Ex19 (L1)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-12</t>
+  </si>
+  <si>
+    <t>Read §5.9 (part 1)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex22(a) (L1)</t>
+  </si>
+  <si>
+    <t>Read §5.9 (part 2)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex22(b) (L1)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex22(c) (L1)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex22(d–f) (L1) (finish Ex22)</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>Read §5.9 (part 1)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex22(a) (L1)</t>
-  </si>
-  <si>
-    <t>Read §5.9 (part 2)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex22(b) (L1)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex22(c) (L1)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex22(d–f) (L1) (finish Ex22)</t>
   </si>
   <si>
     <t>Exercises: Ex24 (L2)</t>
@@ -559,11 +562,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -600,98 +603,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -713,16 +624,45 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -736,6 +676,69 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
@@ -764,6 +767,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -776,7 +809,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -788,37 +851,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -830,49 +893,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -890,61 +911,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -973,6 +976,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -988,34 +1000,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -1038,11 +1028,9 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
+      <top/>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1065,8 +1053,23 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1076,145 +1079,145 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2694,14 +2697,16 @@
         <v>90</v>
       </c>
       <c r="G36" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="13">
+        <f t="shared" si="1"/>
+        <v>46086</v>
+      </c>
+      <c r="I36" s="8"/>
+      <c r="J36" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H36" s="13" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
     <row r="37" spans="1:11">
@@ -2725,14 +2730,16 @@
         <v>90</v>
       </c>
       <c r="G37" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="13">
+        <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
+        <v>46087</v>
+      </c>
+      <c r="I37" s="8"/>
+      <c r="J37" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H37" s="13" t="str">
-        <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
-        <v/>
-      </c>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
     <row r="38" spans="1:11">
@@ -2756,14 +2763,16 @@
         <v>90</v>
       </c>
       <c r="G38" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H38" s="13">
+        <f t="shared" si="3"/>
+        <v>46088</v>
+      </c>
+      <c r="I38" s="8"/>
+      <c r="J38" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H38" s="13" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
     <row r="39" spans="1:11">
@@ -2785,14 +2794,16 @@
         <v>60</v>
       </c>
       <c r="G39" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="13">
+        <f t="shared" si="3"/>
+        <v>46089</v>
+      </c>
+      <c r="I39" s="8"/>
+      <c r="J39" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H39" s="13" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
       <c r="K39" s="8"/>
     </row>
     <row r="40" spans="1:11">
@@ -2814,7 +2825,7 @@
         <v>90</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H40" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2837,13 +2848,13 @@
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F41" s="8">
         <v>60</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H41" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2866,13 +2877,13 @@
       </c>
       <c r="D42" s="8"/>
       <c r="E42" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F42" s="8">
         <v>75</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H42" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2895,13 +2906,13 @@
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H43" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2924,13 +2935,13 @@
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H44" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2953,13 +2964,13 @@
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H45" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2978,17 +2989,17 @@
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H46" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3007,17 +3018,17 @@
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H47" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3036,17 +3047,17 @@
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H48" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3069,13 +3080,13 @@
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H49" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3098,13 +3109,13 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H50" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3127,13 +3138,13 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H51" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3156,13 +3167,13 @@
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H52" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3185,13 +3196,13 @@
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H53" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3214,13 +3225,13 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H54" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3243,13 +3254,13 @@
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H55" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3268,17 +3279,17 @@
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H56" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3335,12 +3346,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
@@ -3349,19 +3360,19 @@
     </row>
     <row r="3" ht="27" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
@@ -3372,10 +3383,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -3391,10 +3402,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3410,10 +3421,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -3429,10 +3440,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3448,10 +3459,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -3467,17 +3478,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -3486,10 +3497,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -3505,10 +3516,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -3524,10 +3535,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
@@ -3543,10 +3554,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3562,10 +3573,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
@@ -3581,10 +3592,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
@@ -3600,10 +3611,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -3619,10 +3630,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
@@ -3638,10 +3649,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3657,17 +3668,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -3676,10 +3687,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
@@ -3695,10 +3706,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
@@ -3714,10 +3725,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
@@ -3733,10 +3744,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
@@ -3752,10 +3763,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
@@ -3771,10 +3782,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
@@ -3790,10 +3801,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
@@ -3809,10 +3820,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3828,10 +3839,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
@@ -3847,10 +3858,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
@@ -3866,10 +3877,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
@@ -3885,10 +3896,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3904,10 +3915,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3923,10 +3934,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3942,17 +3953,17 @@
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -3961,17 +3972,17 @@
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -3980,17 +3991,17 @@
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -3999,17 +4010,17 @@
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -4018,10 +4029,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
@@ -4037,10 +4048,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -4056,10 +4067,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -4075,10 +4086,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -4094,10 +4105,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
@@ -4113,10 +4124,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
@@ -4151,12 +4162,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
@@ -4169,7 +4180,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
@@ -4177,16 +4188,16 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
@@ -4195,11 +4206,11 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4208,7 +4219,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
@@ -4220,16 +4231,16 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>

</xml_diff>

<commit_message>
Chap 5, EX 24
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="179">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -329,13 +329,16 @@
     <t>Exercises: Ex22(d–f) (L1) (finish Ex22)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-13</t>
+  </si>
+  <si>
+    <t>Exercises: Ex24 (L2)</t>
+  </si>
+  <si>
+    <t>Exercises: Ex35 (L2)</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>Exercises: Ex24 (L2)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex35 (L2)</t>
   </si>
   <si>
     <t>Exercises: Ex28 (L2)</t>
@@ -562,11 +565,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -602,6 +605,22 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -609,8 +628,76 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="13"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -625,43 +712,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -669,15 +719,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -685,39 +727,8 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -732,15 +743,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -767,13 +770,85 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -791,13 +866,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -809,13 +878,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -833,55 +920,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -893,61 +950,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -972,15 +975,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1029,8 +1023,41 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1049,40 +1076,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1091,133 +1094,133 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2825,14 +2828,16 @@
         <v>90</v>
       </c>
       <c r="G40" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="13">
+        <f t="shared" si="3"/>
+        <v>46090</v>
+      </c>
+      <c r="I40" s="8"/>
+      <c r="J40" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="H40" s="13" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
     <row r="41" spans="1:11">
@@ -2854,14 +2859,16 @@
         <v>60</v>
       </c>
       <c r="G41" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="13">
+        <f t="shared" si="3"/>
+        <v>46091</v>
+      </c>
+      <c r="I41" s="8"/>
+      <c r="J41" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="H41" s="13" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
     <row r="42" spans="1:11">
@@ -2883,7 +2890,7 @@
         <v>75</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H42" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2906,13 +2913,13 @@
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F43" s="8">
         <v>60</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H43" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2935,13 +2942,13 @@
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F44" s="8">
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H44" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2964,13 +2971,13 @@
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H45" s="13" t="str">
         <f t="shared" si="3"/>
@@ -2989,17 +2996,17 @@
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H46" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3018,17 +3025,17 @@
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F47" s="8">
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H47" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3047,17 +3054,17 @@
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H48" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3080,13 +3087,13 @@
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H49" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3109,13 +3116,13 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H50" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3138,13 +3145,13 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H51" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3167,13 +3174,13 @@
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H52" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3196,13 +3203,13 @@
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H53" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3225,13 +3232,13 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H54" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3254,13 +3261,13 @@
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H55" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3279,17 +3286,17 @@
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H56" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3346,12 +3353,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
@@ -3360,19 +3367,19 @@
     </row>
     <row r="3" ht="27" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
@@ -3383,10 +3390,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -3402,10 +3409,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3421,10 +3428,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -3440,10 +3447,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3459,10 +3466,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -3478,17 +3485,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -3497,10 +3504,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -3516,10 +3523,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -3535,10 +3542,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
@@ -3554,10 +3561,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3573,10 +3580,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
@@ -3592,10 +3599,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
@@ -3611,10 +3618,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -3630,10 +3637,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
@@ -3649,10 +3656,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3668,17 +3675,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -3687,10 +3694,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
@@ -3706,10 +3713,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
@@ -3725,10 +3732,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
@@ -3744,10 +3751,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
@@ -3763,10 +3770,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
@@ -3782,10 +3789,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
@@ -3801,10 +3808,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
@@ -3820,10 +3827,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3839,10 +3846,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
@@ -3858,10 +3865,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
@@ -3877,10 +3884,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
@@ -3896,10 +3903,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3915,10 +3922,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3934,10 +3941,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3953,17 +3960,17 @@
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -3972,17 +3979,17 @@
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -3991,17 +3998,17 @@
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -4010,17 +4017,17 @@
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -4029,10 +4036,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
@@ -4048,10 +4055,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -4067,10 +4074,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -4086,10 +4093,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -4105,10 +4112,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
@@ -4124,10 +4131,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
@@ -4162,12 +4169,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
@@ -4180,7 +4187,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
@@ -4188,16 +4195,16 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
@@ -4206,11 +4213,11 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4219,7 +4226,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
@@ -4231,16 +4238,16 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>

</xml_diff>

<commit_message>
Chap 5, EX 31 (a)-(e)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="183">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -350,22 +350,28 @@
     <t>Exercises: Ex26 (L2)</t>
   </si>
   <si>
+    <t>Exercises: Ex29 (L2)</t>
+  </si>
+  <si>
+    <t>wrap</t>
+  </si>
+  <si>
+    <t>Exercises: Ex32 (L2), Ex33 (L2), Ex34 (L2)</t>
+  </si>
+  <si>
+    <t>Actual done Ex32: 2026-03-17, Ex33, 34: 2026-03-18</t>
+  </si>
+  <si>
+    <t>Exercises: Ex31(a–d) (L2)</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Exercises: Ex31(e–g) (L2)</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>Exercises: Ex29 (L2)</t>
-  </si>
-  <si>
-    <t>wrap</t>
-  </si>
-  <si>
-    <t>Exercises: Ex32 (L2), Ex33 (L2), Ex34 (L2)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex31(a–d) (L2)</t>
-  </si>
-  <si>
-    <t>Exercises: Ex31(e–g) (L2)</t>
   </si>
   <si>
     <t>Exercises: Ex25 (L3) (part 1)</t>
@@ -571,10 +577,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="24">
@@ -611,25 +617,49 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -648,7 +678,39 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -662,31 +724,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
@@ -695,7 +732,7 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -709,25 +746,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -735,21 +755,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -776,37 +782,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -818,43 +830,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -866,49 +842,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -926,19 +860,91 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -950,13 +956,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -985,6 +991,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
@@ -994,17 +1015,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1039,37 +1054,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FFB2B2B2"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1082,16 +1077,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1100,133 +1106,133 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2958,14 +2964,16 @@
         <v>60</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H44" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H44" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46094</v>
       </c>
       <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
+      <c r="J44" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="K44" s="8"/>
     </row>
     <row r="45" spans="1:11">
@@ -2981,23 +2989,25 @@
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F45" s="8">
         <v>60</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H45" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H45" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46095</v>
       </c>
       <c r="I45" s="8"/>
-      <c r="J45" s="8"/>
+      <c r="J45" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" ht="27" spans="1:11">
       <c r="A46" s="11">
         <v>42</v>
       </c>
@@ -3006,24 +3016,26 @@
         <v>46094</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F46" s="8">
         <v>75</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H46" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H46" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46096</v>
       </c>
       <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
+      <c r="J46" s="14" t="s">
+        <v>112</v>
+      </c>
       <c r="K46" s="8"/>
     </row>
     <row r="47" spans="1:11">
@@ -3035,7 +3047,7 @@
         <v>46095</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8" t="s">
@@ -3045,7 +3057,7 @@
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H47" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3064,17 +3076,17 @@
         <v>46096</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H48" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3097,13 +3109,13 @@
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H49" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3126,13 +3138,13 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H50" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3155,13 +3167,13 @@
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F51" s="8">
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H51" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3184,13 +3196,13 @@
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H52" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3213,13 +3225,13 @@
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H53" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3242,13 +3254,13 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H54" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3271,13 +3283,13 @@
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H55" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3296,17 +3308,17 @@
         <v>46104</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H56" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3363,12 +3375,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
@@ -3377,19 +3389,19 @@
     </row>
     <row r="3" ht="27" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
@@ -3400,10 +3412,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -3419,10 +3431,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3438,10 +3450,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -3457,10 +3469,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -3476,10 +3488,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -3495,17 +3507,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -3514,10 +3526,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -3533,10 +3545,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -3552,10 +3564,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
@@ -3571,10 +3583,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3590,10 +3602,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
@@ -3609,10 +3621,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
@@ -3628,10 +3640,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -3647,10 +3659,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
@@ -3666,10 +3678,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3685,17 +3697,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -3704,10 +3716,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
@@ -3723,10 +3735,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
@@ -3742,10 +3754,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
@@ -3761,10 +3773,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
@@ -3780,10 +3792,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
@@ -3799,10 +3811,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
@@ -3818,10 +3830,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
@@ -3837,10 +3849,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3856,10 +3868,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
@@ -3875,10 +3887,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
@@ -3894,10 +3906,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
@@ -3913,10 +3925,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3932,10 +3944,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3951,10 +3963,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3970,17 +3982,17 @@
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
         <v>2026-03-14 – 2026-03-15</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -3989,17 +4001,17 @@
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -4008,17 +4020,17 @@
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -4027,17 +4039,17 @@
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
         <v>2026-03-13</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -4046,10 +4058,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
@@ -4065,10 +4077,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -4084,10 +4096,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -4103,10 +4115,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -4122,10 +4134,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
@@ -4141,10 +4153,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
@@ -4179,12 +4191,12 @@
   <sheetData>
     <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
@@ -4197,7 +4209,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
@@ -4205,29 +4217,29 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4236,7 +4248,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
@@ -4248,16 +4260,16 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>

</xml_diff>

<commit_message>
Chap 5, EX 31 (f)-(g)
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="183">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -365,16 +365,16 @@
     <t>Exercises: Ex31(a–d) (L2)</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>Exercises: Ex31(e–g) (L2)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-24</t>
+  </si>
+  <si>
+    <t>Exercises: Ex25 (L3) (part 1)</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>Exercises: Ex25 (L3) (part 1)</t>
   </si>
   <si>
     <t>Exercises: Ex25 (L3) (part 2) (finish Ex25)</t>
@@ -577,11 +577,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -617,6 +617,42 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -625,8 +661,37 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="13"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -641,44 +706,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -692,17 +722,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <i/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -719,43 +756,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -782,7 +782,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -794,7 +806,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -806,7 +848,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -818,97 +914,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -920,25 +944,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -950,19 +962,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -991,35 +991,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1039,17 +1015,46 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
+      <right style="double">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top style="thin">
+      <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="thin">
+      <bottom style="double">
         <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1069,22 +1074,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1094,145 +1094,145 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -3057,11 +3057,11 @@
         <v>90</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="H47" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H47" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46097</v>
       </c>
       <c r="I47" s="8"/>
       <c r="J47" s="8"/>
@@ -3080,20 +3080,22 @@
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F48" s="8">
         <v>90</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="H48" s="13" t="str">
+        <v>17</v>
+      </c>
+      <c r="H48" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46098</v>
       </c>
       <c r="I48" s="8"/>
-      <c r="J48" s="8"/>
+      <c r="J48" s="8" t="s">
+        <v>115</v>
+      </c>
       <c r="K48" s="8"/>
     </row>
     <row r="49" spans="1:11">
@@ -3109,13 +3111,13 @@
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F49" s="8">
         <v>60</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H49" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3144,7 +3146,7 @@
         <v>60</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H50" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3173,7 +3175,7 @@
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H51" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3202,7 +3204,7 @@
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H52" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3231,7 +3233,7 @@
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H53" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3260,7 +3262,7 @@
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H54" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3289,7 +3291,7 @@
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H55" s="13" t="str">
         <f t="shared" si="3"/>
@@ -3318,7 +3320,7 @@
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H56" s="13" t="str">
         <f t="shared" si="3"/>
@@ -4221,7 +4223,7 @@
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -4230,7 +4232,7 @@
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -4239,7 +4241,7 @@
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -4264,7 +4266,7 @@
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:2">

</xml_diff>

<commit_message>
Chap 5, EX 9,39,40
</commit_message>
<xml_diff>
--- a/Chapter5_Learning_Plan.xlsx
+++ b/Chapter5_Learning_Plan.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_607AB54B5F6E991270EEAF9FEFBB2864F8EEE939" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFBDAAD2-1943-4FA3-BD64-E7E02794A0BD}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="2730" windowWidth="21885" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19935" windowHeight="7785"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Plan" sheetId="1" r:id="rId1"/>
@@ -21,25 +15,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Plan'!$A$4:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercise Map'!$A$3:$F$43</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="188">
   <si>
     <t>Chapter 5 Learning Plan (Resnick: A Probability Path)</t>
   </si>
@@ -393,27 +374,42 @@
     <t>Exercises: Ex25 (L3) (part 1)</t>
   </si>
   <si>
-    <t>Not Started</t>
-  </si>
-  <si>
     <t>Exercises: Ex25 (L3) (part 2) (finish Ex25)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-25</t>
+  </si>
+  <si>
     <t>Exercises: Ex37 (L1)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-27</t>
+  </si>
+  <si>
     <t>Exercises: Ex9 (L2)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-28</t>
+  </si>
+  <si>
     <t>Exercises: Ex39 (L2) (part 1)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-29</t>
+  </si>
+  <si>
     <t>Exercises: Ex39 (L2) (part 2) (finish Ex39)</t>
   </si>
   <si>
+    <t>Actual done: 2026-03-30</t>
+  </si>
+  <si>
     <t>Exercises: Ex40(a–b) (L2)</t>
   </si>
   <si>
+    <t>Actual done: 2026-04-01</t>
+  </si>
+  <si>
     <t>Chapter 5 wrap: 1-page Moves List + confirm all 40 exercises have entries</t>
   </si>
   <si>
@@ -589,20 +585,20 @@
   </si>
   <si>
     <t>C1 Marked Yes</t>
-  </si>
-  <si>
-    <t>Actual done: 2026-03-25</t>
-    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -636,22 +632,151 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
-      <family val="3"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
-      <family val="3"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -670,8 +795,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -694,11 +1005,253 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -718,6 +1271,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -726,21 +1280,66 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -754,7 +1353,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -763,9 +1362,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1050,14 +1646,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K56"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1071,22 +1667,12 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" ht="20.25" spans="1:1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1100,46 +1686,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A4" s="9" t="s">
+    <row r="4" ht="27" spans="1:11">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A5" s="10">
+    <row r="5" spans="1:11">
+      <c r="A5" s="11">
         <v>1</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="12">
         <f t="shared" ref="B5:B36" si="0">IF($B$2="","",$B$2+A5-1)</f>
         <v>46053</v>
       </c>
@@ -1156,7 +1742,7 @@
       <c r="G5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f t="shared" ref="H5:H36" si="1">IF(G5="Done",B5+2,"")</f>
         <v>46055</v>
       </c>
@@ -1168,11 +1754,11 @@
       </c>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A6" s="10">
+    <row r="6" spans="1:11">
+      <c r="A6" s="11">
         <v>2</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="12">
         <f t="shared" si="0"/>
         <v>46054</v>
       </c>
@@ -1189,7 +1775,7 @@
       <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f t="shared" si="1"/>
         <v>46056</v>
       </c>
@@ -1201,11 +1787,11 @@
       </c>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A7" s="10">
+    <row r="7" spans="1:11">
+      <c r="A7" s="11">
         <v>3</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="12">
         <f t="shared" si="0"/>
         <v>46055</v>
       </c>
@@ -1222,7 +1808,7 @@
       <c r="G7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="13">
         <f t="shared" si="1"/>
         <v>46057</v>
       </c>
@@ -1234,11 +1820,11 @@
       </c>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A8" s="10">
+    <row r="8" spans="1:11">
+      <c r="A8" s="11">
         <v>4</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="12">
         <f t="shared" si="0"/>
         <v>46056</v>
       </c>
@@ -1255,7 +1841,7 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="13">
         <f t="shared" si="1"/>
         <v>46058</v>
       </c>
@@ -1267,11 +1853,11 @@
       </c>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A9" s="10">
+    <row r="9" spans="1:11">
+      <c r="A9" s="11">
         <v>5</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="12">
         <f t="shared" si="0"/>
         <v>46057</v>
       </c>
@@ -1288,7 +1874,7 @@
       <c r="G9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="13">
         <f t="shared" si="1"/>
         <v>46059</v>
       </c>
@@ -1300,11 +1886,11 @@
       </c>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A10" s="10">
+    <row r="10" ht="27" spans="1:11">
+      <c r="A10" s="11">
         <v>6</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="12">
         <f t="shared" si="0"/>
         <v>46058</v>
       </c>
@@ -1321,7 +1907,7 @@
       <c r="G10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="13">
         <f t="shared" si="1"/>
         <v>46060</v>
       </c>
@@ -1331,11 +1917,11 @@
       </c>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A11" s="10">
+    <row r="11" spans="1:11">
+      <c r="A11" s="11">
         <v>7</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="12">
         <f t="shared" si="0"/>
         <v>46059</v>
       </c>
@@ -1352,7 +1938,7 @@
       <c r="G11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="13">
         <f t="shared" si="1"/>
         <v>46061</v>
       </c>
@@ -1362,11 +1948,11 @@
       </c>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A12" s="10">
+    <row r="12" spans="1:11">
+      <c r="A12" s="11">
         <v>8</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="12">
         <f t="shared" si="0"/>
         <v>46060</v>
       </c>
@@ -1385,7 +1971,7 @@
       <c r="G12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="13">
         <f t="shared" si="1"/>
         <v>46062</v>
       </c>
@@ -1395,11 +1981,11 @@
       </c>
       <c r="K12" s="8"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A13" s="10">
+    <row r="13" spans="1:11">
+      <c r="A13" s="11">
         <v>9</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="12">
         <f t="shared" si="0"/>
         <v>46061</v>
       </c>
@@ -1418,7 +2004,7 @@
       <c r="G13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="13">
         <f t="shared" si="1"/>
         <v>46063</v>
       </c>
@@ -1428,11 +2014,11 @@
       </c>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A14" s="10">
+    <row r="14" spans="1:11">
+      <c r="A14" s="11">
         <v>10</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="12">
         <f t="shared" si="0"/>
         <v>46062</v>
       </c>
@@ -1449,7 +2035,7 @@
       <c r="G14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="13">
         <f t="shared" si="1"/>
         <v>46064</v>
       </c>
@@ -1459,11 +2045,11 @@
       </c>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A15" s="10">
+    <row r="15" spans="1:11">
+      <c r="A15" s="11">
         <v>11</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="12">
         <f t="shared" si="0"/>
         <v>46063</v>
       </c>
@@ -1480,7 +2066,7 @@
       <c r="G15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="13">
         <f t="shared" si="1"/>
         <v>46065</v>
       </c>
@@ -1492,11 +2078,11 @@
       </c>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A16" s="10">
+    <row r="16" spans="1:11">
+      <c r="A16" s="11">
         <v>12</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="12">
         <f t="shared" si="0"/>
         <v>46064</v>
       </c>
@@ -1513,7 +2099,7 @@
       <c r="G16" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="13">
         <f t="shared" si="1"/>
         <v>46066</v>
       </c>
@@ -1525,11 +2111,11 @@
       </c>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A17" s="10">
+    <row r="17" spans="1:11">
+      <c r="A17" s="11">
         <v>13</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="12">
         <f t="shared" si="0"/>
         <v>46065</v>
       </c>
@@ -1546,7 +2132,7 @@
       <c r="G17" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="13">
         <f t="shared" si="1"/>
         <v>46067</v>
       </c>
@@ -1556,11 +2142,11 @@
       </c>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A18" s="10">
+    <row r="18" ht="27" spans="1:11">
+      <c r="A18" s="11">
         <v>14</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="12">
         <f t="shared" si="0"/>
         <v>46066</v>
       </c>
@@ -1577,7 +2163,7 @@
       <c r="G18" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="13">
         <f t="shared" si="1"/>
         <v>46068</v>
       </c>
@@ -1587,11 +2173,11 @@
       </c>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A19" s="10">
+    <row r="19" spans="1:11">
+      <c r="A19" s="11">
         <v>15</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="12">
         <f t="shared" si="0"/>
         <v>46067</v>
       </c>
@@ -1610,7 +2196,7 @@
       <c r="G19" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="13">
         <f t="shared" si="1"/>
         <v>46069</v>
       </c>
@@ -1620,11 +2206,11 @@
       </c>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A20" s="10">
+    <row r="20" spans="1:11">
+      <c r="A20" s="11">
         <v>16</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="12">
         <f t="shared" si="0"/>
         <v>46068</v>
       </c>
@@ -1641,7 +2227,7 @@
       <c r="G20" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="13">
         <f t="shared" si="1"/>
         <v>46070</v>
       </c>
@@ -1651,11 +2237,11 @@
       </c>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A21" s="10">
-        <v>17</v>
-      </c>
-      <c r="B21" s="11">
+    <row r="21" ht="27" spans="1:11">
+      <c r="A21" s="11">
+        <v>17</v>
+      </c>
+      <c r="B21" s="12">
         <f t="shared" si="0"/>
         <v>46069</v>
       </c>
@@ -1674,7 +2260,7 @@
       <c r="G21" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="13">
         <f t="shared" si="1"/>
         <v>46071</v>
       </c>
@@ -1684,11 +2270,11 @@
       </c>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A22" s="10">
+    <row r="22" spans="1:11">
+      <c r="A22" s="11">
         <v>18</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="12">
         <f t="shared" si="0"/>
         <v>46070</v>
       </c>
@@ -1705,7 +2291,7 @@
       <c r="G22" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="13">
         <f t="shared" si="1"/>
         <v>46072</v>
       </c>
@@ -1715,11 +2301,11 @@
       </c>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A23" s="10">
+    <row r="23" spans="1:11">
+      <c r="A23" s="11">
         <v>19</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="12">
         <f t="shared" si="0"/>
         <v>46071</v>
       </c>
@@ -1736,7 +2322,7 @@
       <c r="G23" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H23" s="12">
+      <c r="H23" s="13">
         <f t="shared" si="1"/>
         <v>46073</v>
       </c>
@@ -1746,11 +2332,11 @@
       </c>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A24" s="10">
+    <row r="24" spans="1:11">
+      <c r="A24" s="11">
         <v>20</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="12">
         <f t="shared" si="0"/>
         <v>46072</v>
       </c>
@@ -1767,7 +2353,7 @@
       <c r="G24" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="13">
         <f t="shared" si="1"/>
         <v>46074</v>
       </c>
@@ -1777,11 +2363,11 @@
       </c>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A25" s="10">
+    <row r="25" spans="1:11">
+      <c r="A25" s="11">
         <v>21</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="12">
         <f t="shared" si="0"/>
         <v>46073</v>
       </c>
@@ -1798,7 +2384,7 @@
       <c r="G25" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H25" s="12">
+      <c r="H25" s="13">
         <f t="shared" si="1"/>
         <v>46075</v>
       </c>
@@ -1808,11 +2394,11 @@
       </c>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A26" s="10">
+    <row r="26" spans="1:11">
+      <c r="A26" s="11">
         <v>22</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="12">
         <f t="shared" si="0"/>
         <v>46074</v>
       </c>
@@ -1831,7 +2417,7 @@
       <c r="G26" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="13">
         <f t="shared" si="1"/>
         <v>46076</v>
       </c>
@@ -1841,11 +2427,11 @@
       </c>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A27" s="10">
+    <row r="27" spans="1:11">
+      <c r="A27" s="11">
         <v>23</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="12">
         <f t="shared" si="0"/>
         <v>46075</v>
       </c>
@@ -1862,7 +2448,7 @@
       <c r="G27" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H27" s="12">
+      <c r="H27" s="13">
         <f t="shared" si="1"/>
         <v>46077</v>
       </c>
@@ -1872,11 +2458,11 @@
       </c>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A28" s="10">
+    <row r="28" spans="1:11">
+      <c r="A28" s="11">
         <v>24</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="12">
         <f t="shared" si="0"/>
         <v>46076</v>
       </c>
@@ -1895,7 +2481,7 @@
       <c r="G28" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="13">
         <f t="shared" si="1"/>
         <v>46078</v>
       </c>
@@ -1905,11 +2491,11 @@
       </c>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A29" s="10">
+    <row r="29" spans="1:11">
+      <c r="A29" s="11">
         <v>25</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="12">
         <f t="shared" si="0"/>
         <v>46077</v>
       </c>
@@ -1926,7 +2512,7 @@
       <c r="G29" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="13">
         <f t="shared" si="1"/>
         <v>46079</v>
       </c>
@@ -1934,11 +2520,11 @@
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A30" s="10">
+    <row r="30" spans="1:11">
+      <c r="A30" s="11">
         <v>26</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="12">
         <f t="shared" si="0"/>
         <v>46078</v>
       </c>
@@ -1955,7 +2541,7 @@
       <c r="G30" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="13">
         <f t="shared" si="1"/>
         <v>46080</v>
       </c>
@@ -1965,11 +2551,11 @@
       </c>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A31" s="10">
+    <row r="31" spans="1:11">
+      <c r="A31" s="11">
         <v>27</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="12">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
@@ -1986,7 +2572,7 @@
       <c r="G31" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="13">
         <f t="shared" si="1"/>
         <v>46081</v>
       </c>
@@ -1996,11 +2582,11 @@
       </c>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A32" s="10">
+    <row r="32" spans="1:11">
+      <c r="A32" s="11">
         <v>28</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="12">
         <f t="shared" si="0"/>
         <v>46080</v>
       </c>
@@ -2017,7 +2603,7 @@
       <c r="G32" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="13">
         <f t="shared" si="1"/>
         <v>46082</v>
       </c>
@@ -2027,11 +2613,11 @@
       </c>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A33" s="10">
+    <row r="33" spans="1:11">
+      <c r="A33" s="11">
         <v>29</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="12">
         <f t="shared" si="0"/>
         <v>46081</v>
       </c>
@@ -2050,7 +2636,7 @@
       <c r="G33" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="12">
+      <c r="H33" s="13">
         <f t="shared" si="1"/>
         <v>46083</v>
       </c>
@@ -2060,11 +2646,11 @@
       </c>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A34" s="10">
+    <row r="34" spans="1:11">
+      <c r="A34" s="11">
         <v>30</v>
       </c>
-      <c r="B34" s="11">
+      <c r="B34" s="12">
         <f t="shared" si="0"/>
         <v>46082</v>
       </c>
@@ -2081,7 +2667,7 @@
       <c r="G34" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H34" s="12">
+      <c r="H34" s="13">
         <f t="shared" si="1"/>
         <v>46084</v>
       </c>
@@ -2091,11 +2677,11 @@
       </c>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A35" s="10">
+    <row r="35" spans="1:11">
+      <c r="A35" s="11">
         <v>31</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="12">
         <f t="shared" si="0"/>
         <v>46083</v>
       </c>
@@ -2112,7 +2698,7 @@
       <c r="G35" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H35" s="12">
+      <c r="H35" s="13">
         <f t="shared" si="1"/>
         <v>46085</v>
       </c>
@@ -2122,11 +2708,11 @@
       </c>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A36" s="10">
+    <row r="36" spans="1:11">
+      <c r="A36" s="11">
         <v>32</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="12">
         <f t="shared" si="0"/>
         <v>46084</v>
       </c>
@@ -2143,7 +2729,7 @@
       <c r="G36" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="12">
+      <c r="H36" s="13">
         <f t="shared" si="1"/>
         <v>46086</v>
       </c>
@@ -2153,11 +2739,11 @@
       </c>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A37" s="10">
+    <row r="37" spans="1:11">
+      <c r="A37" s="11">
         <v>33</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="12">
         <f t="shared" ref="B37:B56" si="2">IF($B$2="","",$B$2+A37-1)</f>
         <v>46085</v>
       </c>
@@ -2176,7 +2762,7 @@
       <c r="G37" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H37" s="12">
+      <c r="H37" s="13">
         <f t="shared" ref="H37:H56" si="3">IF(G37="Done",B37+2,"")</f>
         <v>46087</v>
       </c>
@@ -2186,11 +2772,11 @@
       </c>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A38" s="10">
+    <row r="38" spans="1:11">
+      <c r="A38" s="11">
         <v>34</v>
       </c>
-      <c r="B38" s="11">
+      <c r="B38" s="12">
         <f t="shared" si="2"/>
         <v>46086</v>
       </c>
@@ -2209,7 +2795,7 @@
       <c r="G38" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="13">
         <f t="shared" si="3"/>
         <v>46088</v>
       </c>
@@ -2219,11 +2805,11 @@
       </c>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A39" s="10">
+    <row r="39" spans="1:11">
+      <c r="A39" s="11">
         <v>35</v>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="12">
         <f t="shared" si="2"/>
         <v>46087</v>
       </c>
@@ -2240,7 +2826,7 @@
       <c r="G39" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="12">
+      <c r="H39" s="13">
         <f t="shared" si="3"/>
         <v>46089</v>
       </c>
@@ -2250,11 +2836,11 @@
       </c>
       <c r="K39" s="8"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A40" s="10">
+    <row r="40" spans="1:11">
+      <c r="A40" s="11">
         <v>36</v>
       </c>
-      <c r="B40" s="11">
+      <c r="B40" s="12">
         <f t="shared" si="2"/>
         <v>46088</v>
       </c>
@@ -2271,7 +2857,7 @@
       <c r="G40" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H40" s="12">
+      <c r="H40" s="13">
         <f t="shared" si="3"/>
         <v>46090</v>
       </c>
@@ -2281,11 +2867,11 @@
       </c>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A41" s="10">
+    <row r="41" spans="1:11">
+      <c r="A41" s="11">
         <v>37</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="12">
         <f t="shared" si="2"/>
         <v>46089</v>
       </c>
@@ -2302,7 +2888,7 @@
       <c r="G41" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H41" s="12">
+      <c r="H41" s="13">
         <f t="shared" si="3"/>
         <v>46091</v>
       </c>
@@ -2312,11 +2898,11 @@
       </c>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A42" s="10">
+    <row r="42" spans="1:11">
+      <c r="A42" s="11">
         <v>38</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="12">
         <f t="shared" si="2"/>
         <v>46090</v>
       </c>
@@ -2333,7 +2919,7 @@
       <c r="G42" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H42" s="12">
+      <c r="H42" s="13">
         <f t="shared" si="3"/>
         <v>46092</v>
       </c>
@@ -2343,11 +2929,11 @@
       </c>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A43" s="10">
+    <row r="43" spans="1:11">
+      <c r="A43" s="11">
         <v>39</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="12">
         <f t="shared" si="2"/>
         <v>46091</v>
       </c>
@@ -2364,7 +2950,7 @@
       <c r="G43" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H43" s="12">
+      <c r="H43" s="13">
         <f t="shared" si="3"/>
         <v>46093</v>
       </c>
@@ -2374,11 +2960,11 @@
       </c>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A44" s="10">
+    <row r="44" spans="1:11">
+      <c r="A44" s="11">
         <v>40</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="12">
         <f t="shared" si="2"/>
         <v>46092</v>
       </c>
@@ -2395,7 +2981,7 @@
       <c r="G44" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H44" s="12">
+      <c r="H44" s="13">
         <f t="shared" si="3"/>
         <v>46094</v>
       </c>
@@ -2405,11 +2991,11 @@
       </c>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A45" s="10">
+    <row r="45" spans="1:11">
+      <c r="A45" s="11">
         <v>41</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="12">
         <f t="shared" si="2"/>
         <v>46093</v>
       </c>
@@ -2426,7 +3012,7 @@
       <c r="G45" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H45" s="12">
+      <c r="H45" s="13">
         <f t="shared" si="3"/>
         <v>46095</v>
       </c>
@@ -2436,11 +3022,11 @@
       </c>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A46" s="10">
+    <row r="46" ht="27" spans="1:11">
+      <c r="A46" s="11">
         <v>42</v>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="12">
         <f t="shared" si="2"/>
         <v>46094</v>
       </c>
@@ -2457,7 +3043,7 @@
       <c r="G46" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H46" s="12">
+      <c r="H46" s="13">
         <f t="shared" si="3"/>
         <v>46096</v>
       </c>
@@ -2467,11 +3053,11 @@
       </c>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A47" s="10">
+    <row r="47" spans="1:11">
+      <c r="A47" s="11">
         <v>43</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="12">
         <f t="shared" si="2"/>
         <v>46095</v>
       </c>
@@ -2488,7 +3074,7 @@
       <c r="G47" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H47" s="12">
+      <c r="H47" s="13">
         <f t="shared" si="3"/>
         <v>46097</v>
       </c>
@@ -2496,11 +3082,11 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A48" s="10">
+    <row r="48" spans="1:11">
+      <c r="A48" s="11">
         <v>44</v>
       </c>
-      <c r="B48" s="11">
+      <c r="B48" s="12">
         <f t="shared" si="2"/>
         <v>46096</v>
       </c>
@@ -2517,7 +3103,7 @@
       <c r="G48" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H48" s="12">
+      <c r="H48" s="13">
         <f t="shared" si="3"/>
         <v>46098</v>
       </c>
@@ -2527,11 +3113,11 @@
       </c>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A49" s="10">
+    <row r="49" spans="1:11">
+      <c r="A49" s="11">
         <v>45</v>
       </c>
-      <c r="B49" s="11">
+      <c r="B49" s="12">
         <f t="shared" si="2"/>
         <v>46097</v>
       </c>
@@ -2548,7 +3134,7 @@
       <c r="G49" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H49" s="12">
+      <c r="H49" s="13">
         <f t="shared" si="3"/>
         <v>46099</v>
       </c>
@@ -2556,11 +3142,11 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A50" s="10">
+    <row r="50" spans="1:11">
+      <c r="A50" s="11">
         <v>46</v>
       </c>
-      <c r="B50" s="11">
+      <c r="B50" s="12">
         <f t="shared" si="2"/>
         <v>46098</v>
       </c>
@@ -2569,7 +3155,7 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F50" s="8">
         <v>60</v>
@@ -2577,21 +3163,21 @@
       <c r="G50" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H50" s="13">
         <f t="shared" si="3"/>
         <v>46100</v>
       </c>
       <c r="I50" s="8"/>
-      <c r="J50" s="16" t="s">
-        <v>183</v>
+      <c r="J50" s="14" t="s">
+        <v>118</v>
       </c>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A51" s="10">
+    <row r="51" spans="1:11">
+      <c r="A51" s="11">
         <v>47</v>
       </c>
-      <c r="B51" s="11">
+      <c r="B51" s="12">
         <f t="shared" si="2"/>
         <v>46099</v>
       </c>
@@ -2606,21 +3192,23 @@
         <v>90</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H51" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H51" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46101</v>
       </c>
       <c r="I51" s="8"/>
-      <c r="J51" s="8"/>
+      <c r="J51" s="14" t="s">
+        <v>120</v>
+      </c>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A52" s="10">
+    <row r="52" spans="1:11">
+      <c r="A52" s="11">
         <v>48</v>
       </c>
-      <c r="B52" s="11">
+      <c r="B52" s="12">
         <f t="shared" si="2"/>
         <v>46100</v>
       </c>
@@ -2629,27 +3217,29 @@
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F52" s="8">
         <v>60</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H52" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H52" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46102</v>
       </c>
       <c r="I52" s="8"/>
-      <c r="J52" s="8"/>
+      <c r="J52" s="14" t="s">
+        <v>122</v>
+      </c>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A53" s="10">
+    <row r="53" spans="1:11">
+      <c r="A53" s="11">
         <v>49</v>
       </c>
-      <c r="B53" s="11">
+      <c r="B53" s="12">
         <f t="shared" si="2"/>
         <v>46101</v>
       </c>
@@ -2658,27 +3248,29 @@
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F53" s="8">
         <v>90</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H53" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H53" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46103</v>
       </c>
       <c r="I53" s="8"/>
-      <c r="J53" s="8"/>
+      <c r="J53" s="14" t="s">
+        <v>124</v>
+      </c>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A54" s="10">
+    <row r="54" spans="1:11">
+      <c r="A54" s="11">
         <v>50</v>
       </c>
-      <c r="B54" s="11">
+      <c r="B54" s="12">
         <f t="shared" si="2"/>
         <v>46102</v>
       </c>
@@ -2687,27 +3279,29 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F54" s="8">
         <v>90</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H54" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H54" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46104</v>
       </c>
       <c r="I54" s="8"/>
-      <c r="J54" s="8"/>
+      <c r="J54" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A55" s="10">
+    <row r="55" spans="1:11">
+      <c r="A55" s="11">
         <v>51</v>
       </c>
-      <c r="B55" s="11">
+      <c r="B55" s="12">
         <f t="shared" si="2"/>
         <v>46103</v>
       </c>
@@ -2716,27 +3310,29 @@
       </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F55" s="8">
         <v>60</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H55" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H55" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46105</v>
       </c>
       <c r="I55" s="8"/>
-      <c r="J55" s="8"/>
+      <c r="J55" s="14" t="s">
+        <v>128</v>
+      </c>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" spans="1:11" ht="27" x14ac:dyDescent="0.15">
-      <c r="A56" s="10">
+    <row r="56" ht="27" spans="1:11">
+      <c r="A56" s="11">
         <v>52</v>
       </c>
-      <c r="B56" s="11">
+      <c r="B56" s="12">
         <f t="shared" si="2"/>
         <v>46104</v>
       </c>
@@ -2745,55 +3341,58 @@
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F56" s="8">
         <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H56" s="12" t="str">
+        <v>17</v>
+      </c>
+      <c r="H56" s="13">
         <f t="shared" si="3"/>
-        <v/>
+        <v>46106</v>
       </c>
       <c r="I56" s="8"/>
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K56" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:K56">
+    <extLst/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="A5:K56">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G5="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>$G5="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>$G5="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="G5:G56" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="G5:G56">
       <formula1>"Not Started,In Progress,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I5:I56" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I5:I56">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2803,54 +3402,49 @@
     <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="1" ht="18.75" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B2" s="6">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="3" ht="27" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6">
       <c r="A4" s="8">
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+2-1,"yyyy-mm-dd"))</f>
@@ -2861,15 +3455,15 @@
       </c>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6">
       <c r="A5" s="8">
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2880,15 +3474,15 @@
       </c>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6">
       <c r="A6" s="8">
         <v>3</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+3-1,"yyyy-mm-dd"))</f>
@@ -2899,15 +3493,15 @@
       </c>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6">
       <c r="A7" s="8">
         <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+1-1,"yyyy-mm-dd"))</f>
@@ -2918,15 +3512,15 @@
       </c>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="8" ht="27" spans="1:6">
       <c r="A8" s="8">
         <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+4-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+5-1,"yyyy-mm-dd"))</f>
@@ -2937,34 +3531,34 @@
       </c>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="9" ht="27" spans="1:6">
       <c r="A9" s="8">
         <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D9" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+6-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+16-1,"yyyy-mm-dd"))</f>
         <v>2026-02-05 – 2026-02-15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:6">
       <c r="A10" s="8">
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D10" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+9-1,"yyyy-mm-dd"))</f>
@@ -2975,15 +3569,15 @@
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:6">
       <c r="A11" s="8">
         <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D11" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+10-1,"yyyy-mm-dd"))</f>
@@ -2994,15 +3588,15 @@
       </c>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:6">
       <c r="A12" s="8">
         <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D12" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+48-1,"yyyy-mm-dd"))</f>
@@ -3013,15 +3607,15 @@
       </c>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:6">
       <c r="A13" s="8">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D13" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+7-1,"yyyy-mm-dd"))</f>
@@ -3032,15 +3626,15 @@
       </c>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:6">
       <c r="A14" s="8">
         <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D14" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+31-1,"yyyy-mm-dd"))</f>
@@ -3051,15 +3645,15 @@
       </c>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="15" ht="27" spans="1:6">
       <c r="A15" s="8">
         <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D15" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+25-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+26-1,"yyyy-mm-dd"))</f>
@@ -3070,15 +3664,15 @@
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:6">
       <c r="A16" s="8">
         <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D16" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+11-1,"yyyy-mm-dd"))</f>
@@ -3089,15 +3683,15 @@
       </c>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:6">
       <c r="A17" s="8">
         <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D17" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+17-1,"yyyy-mm-dd"))</f>
@@ -3108,15 +3702,15 @@
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:6">
       <c r="A18" s="8">
         <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D18" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+14-1,"yyyy-mm-dd"))</f>
@@ -3127,34 +3721,34 @@
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="19" ht="27" spans="1:6">
       <c r="A19" s="8">
         <v>16</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D19" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+22-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+30-1,"yyyy-mm-dd"))</f>
         <v>2026-02-21 – 2026-03-01</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:6">
       <c r="A20" s="8">
         <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D20" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+27-1,"yyyy-mm-dd"))</f>
@@ -3165,15 +3759,15 @@
       </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:6">
       <c r="A21" s="8">
         <v>18</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D21" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+23-1,"yyyy-mm-dd"))</f>
@@ -3184,15 +3778,15 @@
       </c>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:6">
       <c r="A22" s="8">
         <v>19</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D22" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+32-1,"yyyy-mm-dd"))</f>
@@ -3203,15 +3797,15 @@
       </c>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="23" ht="27" spans="1:6">
       <c r="A23" s="8">
         <v>20</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D23" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+18-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+20-1,"yyyy-mm-dd"))</f>
@@ -3222,15 +3816,15 @@
       </c>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:6">
       <c r="A24" s="8">
         <v>21</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D24" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+21-1,"yyyy-mm-dd"))</f>
@@ -3241,15 +3835,15 @@
       </c>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="25" ht="27" spans="1:6">
       <c r="A25" s="8">
         <v>22</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D25" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+33-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+36-1,"yyyy-mm-dd"))</f>
@@ -3260,15 +3854,15 @@
       </c>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:6">
       <c r="A26" s="8">
         <v>23</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D26" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+24-1,"yyyy-mm-dd"))</f>
@@ -3279,15 +3873,15 @@
       </c>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:6">
       <c r="A27" s="8">
         <v>24</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D27" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+37-1,"yyyy-mm-dd"))</f>
@@ -3298,15 +3892,15 @@
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="28" ht="27" spans="1:6">
       <c r="A28" s="8">
         <v>25</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D28" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+45-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+46-1,"yyyy-mm-dd"))</f>
@@ -3317,15 +3911,15 @@
       </c>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:6">
       <c r="A29" s="8">
         <v>26</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D29" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+40-1,"yyyy-mm-dd"))</f>
@@ -3336,15 +3930,15 @@
       </c>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:6">
       <c r="A30" s="8">
         <v>27</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D30" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+28-1,"yyyy-mm-dd"))</f>
@@ -3355,15 +3949,15 @@
       </c>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:6">
       <c r="A31" s="8">
         <v>28</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D31" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+39-1,"yyyy-mm-dd"))</f>
@@ -3374,15 +3968,15 @@
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:6">
       <c r="A32" s="8">
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D32" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+41-1,"yyyy-mm-dd"))</f>
@@ -3393,15 +3987,15 @@
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:6">
       <c r="A33" s="8">
         <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D33" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+12-1,"yyyy-mm-dd"))</f>
@@ -3412,15 +4006,15 @@
       </c>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="34" ht="27" spans="1:6">
       <c r="A34" s="8">
         <v>31</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D34" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+43-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+44-1,"yyyy-mm-dd"))</f>
@@ -3431,15 +4025,15 @@
       </c>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:6">
       <c r="A35" s="8">
         <v>32</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D35" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
@@ -3450,15 +4044,15 @@
       </c>
       <c r="F35" s="8"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:6">
       <c r="A36" s="8">
         <v>33</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D36" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
@@ -3469,15 +4063,15 @@
       </c>
       <c r="F36" s="8"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:6">
       <c r="A37" s="8">
         <v>34</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D37" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+42-1,"yyyy-mm-dd"))</f>
@@ -3488,15 +4082,15 @@
       </c>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:6">
       <c r="A38" s="8">
         <v>35</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D38" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+38-1,"yyyy-mm-dd"))</f>
@@ -3507,15 +4101,15 @@
       </c>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:6">
       <c r="A39" s="8">
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D39" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+13-1,"yyyy-mm-dd"))</f>
@@ -3526,15 +4120,15 @@
       </c>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:6">
       <c r="A40" s="8">
         <v>37</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D40" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+47-1,"yyyy-mm-dd"))</f>
@@ -3545,15 +4139,15 @@
       </c>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:6">
       <c r="A41" s="8">
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D41" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+8-1,"yyyy-mm-dd"))</f>
@@ -3564,15 +4158,15 @@
       </c>
       <c r="F41" s="8"/>
     </row>
-    <row r="42" spans="1:6" ht="27" x14ac:dyDescent="0.15">
+    <row r="42" ht="27" spans="1:6">
       <c r="A42" s="8">
         <v>39</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D42" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+49-1,"yyyy-mm-dd")&amp;" – "&amp;TEXT($B$2+50-1,"yyyy-mm-dd"))</f>
@@ -3583,15 +4177,15 @@
       </c>
       <c r="F42" s="8"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:6">
       <c r="A43" s="8">
         <v>40</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D43" s="8" t="str">
         <f>IF($B$2="","",TEXT($B$2+51-1,"yyyy-mm-dd"))</f>
@@ -3603,105 +4197,108 @@
       <c r="F43" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F43" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:F43">
+    <extLst/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="18.75" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B3" s="3">
         <f>'Daily Plan'!B2</f>
         <v>46053</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:2">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B5" s="4">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Done")</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"In Progress")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Daily Plan'!G5:G56,"Not Started")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B10" s="4">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Daily Plan'!H5:H56,"&gt;0")</f>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B13" s="4">
         <f>COUNTIF('Daily Plan'!I5:I56,"Yes")</f>
@@ -3709,8 +4306,8 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>